<commit_message>
Add PR VCOM and External Availability columns to mother sheet template and update synchronization logic
</commit_message>
<xml_diff>
--- a/original_format/00 PR_recalculation_APRL.xlsx
+++ b/original_format/00 PR_recalculation_APRL.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\S01\get\2025.01 Mazara 01 A2A\03 - REPORT\Report\09 Testing\PR Calculation automation\original_format\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F9B91A-6FF7-41F5-8D54-20ECC1716594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77932A00-71C1-4946-B344-78BF3E058507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
     <author>Utente</author>
   </authors>
   <commentList>
-    <comment ref="T6" authorId="0" shapeId="0" xr:uid="{2FB631FE-7B5E-43DD-B31B-4C74D1CA6B64}">
+    <comment ref="V6" authorId="0" shapeId="0" xr:uid="{2FB631FE-7B5E-43DD-B31B-4C74D1CA6B64}">
       <text>
         <r>
           <rPr>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Dati</t>
   </si>
@@ -213,6 +213,13 @@
   </si>
   <si>
     <t>PR calculation every day</t>
+  </si>
+  <si>
+    <t>PR VCOM</t>
+  </si>
+  <si>
+    <t>External Availability
+[%]</t>
   </si>
 </sst>
 </file>
@@ -279,7 +286,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -558,11 +565,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -587,9 +609,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -609,13 +628,475 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="88">
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+  <dxfs count="91">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color auto="1"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color auto="1"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="medium">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="medium">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
           <color indexed="64"/>
         </left>
@@ -628,14 +1109,11 @@
         <bottom style="medium">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
           <color indexed="64"/>
         </left>
@@ -648,994 +1126,72 @@
         <bottom style="medium">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
         </left>
-        <right style="medium">
-          <color indexed="64"/>
+        <right style="thin">
+          <color auto="1"/>
         </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
         </left>
-        <right style="medium">
-          <color indexed="64"/>
+        <right style="thin">
+          <color auto="1"/>
         </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
         </left>
-        <right style="medium">
-          <color indexed="64"/>
+        <right style="thin">
+          <color auto="1"/>
         </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
         </left>
-        <right style="medium">
-          <color indexed="64"/>
+        <right style="thin">
+          <color auto="1"/>
         </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-        <horizontal/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.000"/>
       <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
+        <left/>
         <right style="thin">
           <color auto="1"/>
         </right>
@@ -1657,6 +1213,23 @@
       </fill>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <top style="thin">
           <color auto="1"/>
@@ -1994,6 +1567,196 @@
         <horizontal style="thin">
           <color auto="1"/>
         </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -2390,56 +2153,62 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TabellaAPRL2026" displayName="TabellaAPRL2026" ref="A4:AR35" headerRowCount="0" totalsRowCount="1">
-  <tableColumns count="44">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Colonna1" totalsRowDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{B14D2040-0C85-4ABB-B9F2-DB214B494F99}" name="Colonna4" dataDxfId="87" totalsRowDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{6146493F-E789-4F9A-A367-EE09E8A74459}" name="Colonna11" dataDxfId="86" totalsRowDxfId="41"/>
-    <tableColumn id="4" xr3:uid="{50DD95C4-E191-4573-9275-92130C5D20B6}" name="Colonna12" totalsRowFunction="custom" dataDxfId="85" totalsRowDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TabellaAPRL2026" displayName="TabellaAPRL2026" ref="A4:AT35" headerRowCount="0" totalsRowCount="1">
+  <tableColumns count="46">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Colonna1"/>
+    <tableColumn id="2" xr3:uid="{B14D2040-0C85-4ABB-B9F2-DB214B494F99}" name="Colonna4" dataDxfId="90" totalsRowDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{6146493F-E789-4F9A-A367-EE09E8A74459}" name="Colonna11" dataDxfId="89" totalsRowDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{50DD95C4-E191-4573-9275-92130C5D20B6}" name="Colonna12" totalsRowFunction="custom" dataDxfId="88" totalsRowDxfId="42">
       <totalsRowFormula>AVERAGE(D5:D34)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{811DB1BF-4766-44EA-92AC-DE12BBC5C210}" name="Colonna7" totalsRowFunction="custom" dataDxfId="84" totalsRowDxfId="39">
+    <tableColumn id="5" xr3:uid="{811DB1BF-4766-44EA-92AC-DE12BBC5C210}" name="Colonna7" totalsRowFunction="custom" dataDxfId="87" totalsRowDxfId="41">
       <totalsRowFormula>AVERAGE(E5:E34)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{5F7D80EF-8BAA-4131-9F02-2B47B9B4D5BA}" name="Colonna13" dataDxfId="83" totalsRowDxfId="38"/>
-    <tableColumn id="7" xr3:uid="{55D2D573-983E-4C5B-9C48-1BACCA393A88}" name="Colonna14" dataDxfId="82" totalsRowDxfId="37"/>
-    <tableColumn id="8" xr3:uid="{7F240FDF-A189-4AF5-8F29-DEEFB888A9A0}" name="Colonna15" dataDxfId="81" totalsRowDxfId="36"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Colonna24" dataDxfId="80" totalsRowDxfId="35"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Colonna31" dataDxfId="53" totalsRowDxfId="34"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Colonna32" dataDxfId="52" totalsRowDxfId="33"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Colonna33" dataDxfId="51" totalsRowDxfId="32"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colonna34" dataDxfId="50" totalsRowDxfId="31"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Colonna35" dataDxfId="49" totalsRowDxfId="30"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Colonna36" dataDxfId="48" totalsRowDxfId="29"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Colonna37" dataDxfId="47" totalsRowDxfId="28"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Colonna3" dataDxfId="46" totalsRowDxfId="27"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Colonna17" dataDxfId="45" totalsRowDxfId="26"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Colonna19" dataDxfId="44" totalsRowDxfId="25"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Colonna20" dataDxfId="79" totalsRowDxfId="24"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Colonna39" dataDxfId="78" totalsRowDxfId="23"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Colonna40" dataDxfId="77" totalsRowDxfId="22"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Colonna41" dataDxfId="76" totalsRowDxfId="21"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Colonna42" dataDxfId="75" totalsRowDxfId="20"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Colonna43" dataDxfId="74" totalsRowDxfId="19"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Colonna44" dataDxfId="73" totalsRowDxfId="18"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Colonna45" dataDxfId="72" totalsRowDxfId="17"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="Colonna46" dataDxfId="71" totalsRowDxfId="16"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="Colonna38" dataDxfId="70" totalsRowDxfId="15"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Colonna2" dataDxfId="69" totalsRowDxfId="14"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Colonna5" dataDxfId="68" totalsRowDxfId="13"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Colonna6" dataDxfId="67" totalsRowDxfId="12"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="Colonna54" dataDxfId="66" totalsRowDxfId="11"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="Colonna55" dataDxfId="65" totalsRowDxfId="10"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0000-000030000000}" name="Colonna56" dataDxfId="64" totalsRowDxfId="9"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0000-000031000000}" name="Colonna57" dataDxfId="63" totalsRowDxfId="8"/>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0000-000032000000}" name="Colonna58" dataDxfId="62" totalsRowDxfId="7"/>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0000-000033000000}" name="Colonna59" dataDxfId="61" totalsRowDxfId="6"/>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0000-000034000000}" name="Colonna60" dataDxfId="60" totalsRowDxfId="5"/>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0000-000035000000}" name="Colonna61" dataDxfId="59" totalsRowDxfId="4"/>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0000-000036000000}" name="Colonna50" dataDxfId="58" totalsRowDxfId="3"/>
-    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0000-000037000000}" name="Colonna51" dataDxfId="57" totalsRowDxfId="2"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0000-000038000000}" name="Colonna52" dataDxfId="56" totalsRowDxfId="1"/>
-    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0000-000039000000}" name="Colonna53" dataDxfId="55" totalsRowDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{FCEE7969-4D4B-407C-97A5-5796C7281693}" name="Colonna9" totalsRowFunction="custom" dataDxfId="45" totalsRowDxfId="40">
+      <totalsRowFormula>AVERAGE(F5:F34)</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{A4FE1C65-5D9A-47C5-8BF7-1183770FC023}" name="Colonna8" totalsRowFunction="custom" dataDxfId="47" totalsRowDxfId="39">
+      <totalsRowFormula>SUMIF(G5:G34,"&lt;&gt;100")/COUNTIF(G5:G34,"&lt;&gt;100")</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{5F7D80EF-8BAA-4131-9F02-2B47B9B4D5BA}" name="Colonna13" dataDxfId="86" totalsRowDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{55D2D573-983E-4C5B-9C48-1BACCA393A88}" name="Colonna14" dataDxfId="85" totalsRowDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{7F240FDF-A189-4AF5-8F29-DEEFB888A9A0}" name="Colonna15" dataDxfId="84" totalsRowDxfId="36"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Colonna24" dataDxfId="83" totalsRowDxfId="35"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Colonna31" dataDxfId="82" totalsRowDxfId="34"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Colonna32" dataDxfId="81" totalsRowDxfId="33"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Colonna33" dataDxfId="80" totalsRowDxfId="32"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colonna34" dataDxfId="79" totalsRowDxfId="31"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Colonna35" dataDxfId="78" totalsRowDxfId="30"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Colonna36" dataDxfId="77" totalsRowDxfId="29"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Colonna37" dataDxfId="76" totalsRowDxfId="28"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Colonna3" dataDxfId="75" totalsRowDxfId="27"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Colonna17" dataDxfId="74" totalsRowDxfId="26"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Colonna19" dataDxfId="73" totalsRowDxfId="25"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Colonna20" dataDxfId="72" totalsRowDxfId="24"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Colonna39" dataDxfId="71" totalsRowDxfId="23"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Colonna40" dataDxfId="70" totalsRowDxfId="22"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Colonna41" dataDxfId="69" totalsRowDxfId="21"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Colonna42" dataDxfId="68" totalsRowDxfId="20"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Colonna43" dataDxfId="67" totalsRowDxfId="19"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Colonna44" dataDxfId="66" totalsRowDxfId="18"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Colonna45" dataDxfId="65" totalsRowDxfId="17"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="Colonna46" dataDxfId="64" totalsRowDxfId="16"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="Colonna38" dataDxfId="63" totalsRowDxfId="15"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Colonna2" dataDxfId="62" totalsRowDxfId="14"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Colonna5" dataDxfId="61" totalsRowDxfId="13"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Colonna6" dataDxfId="60" totalsRowDxfId="12"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="Colonna54" dataDxfId="59" totalsRowDxfId="11"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="Colonna55" dataDxfId="58" totalsRowDxfId="10"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0000-000030000000}" name="Colonna56" dataDxfId="57" totalsRowDxfId="9"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0000-000031000000}" name="Colonna57" dataDxfId="56" totalsRowDxfId="8"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0000-000032000000}" name="Colonna58" dataDxfId="55" totalsRowDxfId="7"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0000-000033000000}" name="Colonna59" dataDxfId="54" totalsRowDxfId="6"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0000-000034000000}" name="Colonna60" dataDxfId="53" totalsRowDxfId="5"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0000-000035000000}" name="Colonna61" dataDxfId="52" totalsRowDxfId="4"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0000-000036000000}" name="Colonna50" dataDxfId="51" totalsRowDxfId="3"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0000-000037000000}" name="Colonna51" dataDxfId="50" totalsRowDxfId="2"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0000-000038000000}" name="Colonna52" dataDxfId="49" totalsRowDxfId="1"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0000-000039000000}" name="Colonna53" dataDxfId="48" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2621,207 +2390,218 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR35"/>
+  <dimension ref="A1:AT35"/>
   <sheetFormatPr defaultColWidth="13.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:44" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:46" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
-      <c r="S1" s="20"/>
-      <c r="T1" s="20"/>
-      <c r="U1" s="20"/>
-      <c r="V1" s="20"/>
-      <c r="W1" s="20"/>
-      <c r="X1" s="20"/>
-      <c r="Y1" s="20"/>
-      <c r="Z1" s="20"/>
-      <c r="AA1" s="20"/>
-      <c r="AB1" s="20"/>
-      <c r="AC1" s="20"/>
-      <c r="AD1" s="20"/>
-      <c r="AE1" s="20"/>
-      <c r="AF1" s="20"/>
-      <c r="AG1" s="20"/>
-      <c r="AH1" s="20"/>
-      <c r="AI1" s="20"/>
-      <c r="AJ1" s="20"/>
-      <c r="AK1" s="20"/>
-      <c r="AL1" s="20"/>
-      <c r="AM1" s="20"/>
-      <c r="AN1" s="20"/>
-      <c r="AO1" s="20"/>
-      <c r="AP1" s="20"/>
-      <c r="AQ1" s="20"/>
-      <c r="AR1" s="20"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="29"/>
+      <c r="V1" s="29"/>
+      <c r="W1" s="29"/>
+      <c r="X1" s="29"/>
+      <c r="Y1" s="29"/>
+      <c r="Z1" s="29"/>
+      <c r="AA1" s="29"/>
+      <c r="AB1" s="29"/>
+      <c r="AC1" s="29"/>
+      <c r="AD1" s="29"/>
+      <c r="AE1" s="29"/>
+      <c r="AF1" s="29"/>
+      <c r="AG1" s="29"/>
+      <c r="AH1" s="29"/>
+      <c r="AI1" s="29"/>
+      <c r="AJ1" s="29"/>
+      <c r="AK1" s="29"/>
+      <c r="AL1" s="29"/>
+      <c r="AM1" s="29"/>
+      <c r="AN1" s="29"/>
+      <c r="AO1" s="29"/>
+      <c r="AP1" s="29"/>
+      <c r="AQ1" s="29"/>
+      <c r="AR1" s="29"/>
+      <c r="AS1" s="29"/>
+      <c r="AT1" s="29"/>
     </row>
-    <row r="2" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:44" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:44" s="1" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:46" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:46" s="1" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="E4" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="I4" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="H4" s="28" t="s">
+      <c r="J4" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="I4" s="29" t="s">
+      <c r="K4" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="L4" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="K4" s="25" t="s">
+      <c r="M4" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="25" t="s">
+      <c r="N4" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="25" t="s">
+      <c r="O4" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="25" t="s">
+      <c r="P4" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="25" t="s">
+      <c r="Q4" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="P4" s="25" t="s">
+      <c r="R4" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="Q4" s="25" t="s">
+      <c r="S4" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="R4" s="25" t="s">
+      <c r="T4" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="S4" s="25" t="s">
+      <c r="U4" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="T4" s="28" t="s">
+      <c r="V4" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="U4" s="29" t="s">
+      <c r="W4" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="V4" s="25" t="s">
+      <c r="X4" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="W4" s="25" t="s">
+      <c r="Y4" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="X4" s="25" t="s">
+      <c r="Z4" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="Y4" s="25" t="s">
+      <c r="AA4" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="Z4" s="25" t="s">
+      <c r="AB4" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="AA4" s="25" t="s">
+      <c r="AC4" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="AB4" s="25" t="s">
+      <c r="AD4" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="AC4" s="25" t="s">
+      <c r="AE4" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="AD4" s="25" t="s">
+      <c r="AF4" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="AE4" s="25" t="s">
+      <c r="AG4" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="AF4" s="28" t="s">
+      <c r="AH4" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="AG4" s="29" t="s">
+      <c r="AI4" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="AH4" s="25" t="s">
+      <c r="AJ4" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="AI4" s="25" t="s">
+      <c r="AK4" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="AJ4" s="25" t="s">
+      <c r="AL4" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="AK4" s="25" t="s">
+      <c r="AM4" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="AL4" s="25" t="s">
+      <c r="AN4" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="AM4" s="25" t="s">
+      <c r="AO4" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="AN4" s="25" t="s">
+      <c r="AP4" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="AO4" s="25" t="s">
+      <c r="AQ4" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="AP4" s="25" t="s">
+      <c r="AR4" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="AQ4" s="25" t="s">
+      <c r="AS4" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="AR4" s="28" t="s">
+      <c r="AT4" s="27" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
         <v>46113</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
-      <c r="D5" s="21"/>
+      <c r="D5" s="20"/>
       <c r="E5" s="10"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H5" s="21"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="23"/>
       <c r="L5" s="10"/>
       <c r="M5" s="10"/>
       <c r="N5" s="10"/>
@@ -2830,10 +2610,10 @@
       <c r="Q5" s="10"/>
       <c r="R5" s="10"/>
       <c r="S5" s="10"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="24"/>
-      <c r="V5" s="10"/>
-      <c r="W5" s="10"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="21"/>
+      <c r="W5" s="23"/>
       <c r="X5" s="10"/>
       <c r="Y5" s="10"/>
       <c r="Z5" s="10"/>
@@ -2842,10 +2622,10 @@
       <c r="AC5" s="10"/>
       <c r="AD5" s="10"/>
       <c r="AE5" s="10"/>
-      <c r="AF5" s="22"/>
-      <c r="AG5" s="24"/>
-      <c r="AH5" s="10"/>
-      <c r="AI5" s="10"/>
+      <c r="AF5" s="10"/>
+      <c r="AG5" s="10"/>
+      <c r="AH5" s="21"/>
+      <c r="AI5" s="23"/>
       <c r="AJ5" s="10"/>
       <c r="AK5" s="10"/>
       <c r="AL5" s="10"/>
@@ -2854,9 +2634,11 @@
       <c r="AO5" s="10"/>
       <c r="AP5" s="10"/>
       <c r="AQ5" s="10"/>
-      <c r="AR5" s="22"/>
+      <c r="AR5" s="10"/>
+      <c r="AS5" s="10"/>
+      <c r="AT5" s="21"/>
     </row>
-    <row r="6" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>46114</v>
       </c>
@@ -2865,11 +2647,14 @@
       <c r="D6" s="4"/>
       <c r="E6" s="2"/>
       <c r="F6" s="3"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
+      <c r="G6" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="6"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -2878,10 +2663,10 @@
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="6"/>
-      <c r="V6" s="2"/>
-      <c r="W6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="6"/>
       <c r="X6" s="2"/>
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
@@ -2890,10 +2675,10 @@
       <c r="AC6" s="2"/>
       <c r="AD6" s="2"/>
       <c r="AE6" s="2"/>
-      <c r="AF6" s="3"/>
-      <c r="AG6" s="6"/>
-      <c r="AH6" s="2"/>
-      <c r="AI6" s="2"/>
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="3"/>
+      <c r="AI6" s="6"/>
       <c r="AJ6" s="2"/>
       <c r="AK6" s="2"/>
       <c r="AL6" s="2"/>
@@ -2902,9 +2687,11 @@
       <c r="AO6" s="2"/>
       <c r="AP6" s="2"/>
       <c r="AQ6" s="2"/>
-      <c r="AR6" s="3"/>
+      <c r="AR6" s="2"/>
+      <c r="AS6" s="2"/>
+      <c r="AT6" s="3"/>
     </row>
-    <row r="7" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>46115</v>
       </c>
@@ -2913,11 +2700,14 @@
       <c r="D7" s="4"/>
       <c r="E7" s="2"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
+      <c r="G7" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="6"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -2926,10 +2716,10 @@
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="6"/>
-      <c r="V7" s="2"/>
-      <c r="W7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="6"/>
       <c r="X7" s="2"/>
       <c r="Y7" s="2"/>
       <c r="Z7" s="2"/>
@@ -2938,10 +2728,10 @@
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
       <c r="AE7" s="2"/>
-      <c r="AF7" s="3"/>
-      <c r="AG7" s="6"/>
-      <c r="AH7" s="2"/>
-      <c r="AI7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="3"/>
+      <c r="AI7" s="6"/>
       <c r="AJ7" s="2"/>
       <c r="AK7" s="2"/>
       <c r="AL7" s="2"/>
@@ -2950,9 +2740,11 @@
       <c r="AO7" s="2"/>
       <c r="AP7" s="2"/>
       <c r="AQ7" s="2"/>
-      <c r="AR7" s="3"/>
+      <c r="AR7" s="2"/>
+      <c r="AS7" s="2"/>
+      <c r="AT7" s="3"/>
     </row>
-    <row r="8" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
         <v>46116</v>
       </c>
@@ -2961,11 +2753,14 @@
       <c r="D8" s="4"/>
       <c r="E8" s="2"/>
       <c r="F8" s="3"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
+      <c r="G8" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H8" s="3"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="6"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
@@ -2974,10 +2769,10 @@
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
-      <c r="T8" s="3"/>
-      <c r="U8" s="6"/>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="6"/>
       <c r="X8" s="2"/>
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
@@ -2986,10 +2781,10 @@
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
       <c r="AE8" s="2"/>
-      <c r="AF8" s="3"/>
-      <c r="AG8" s="6"/>
-      <c r="AH8" s="2"/>
-      <c r="AI8" s="2"/>
+      <c r="AF8" s="2"/>
+      <c r="AG8" s="2"/>
+      <c r="AH8" s="3"/>
+      <c r="AI8" s="6"/>
       <c r="AJ8" s="2"/>
       <c r="AK8" s="2"/>
       <c r="AL8" s="2"/>
@@ -2998,9 +2793,11 @@
       <c r="AO8" s="2"/>
       <c r="AP8" s="2"/>
       <c r="AQ8" s="2"/>
-      <c r="AR8" s="3"/>
+      <c r="AR8" s="2"/>
+      <c r="AS8" s="2"/>
+      <c r="AT8" s="3"/>
     </row>
-    <row r="9" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>46117</v>
       </c>
@@ -3009,11 +2806,14 @@
       <c r="D9" s="4"/>
       <c r="E9" s="2"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
+      <c r="G9" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H9" s="3"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="6"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
@@ -3022,10 +2822,10 @@
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
       <c r="S9" s="2"/>
-      <c r="T9" s="3"/>
-      <c r="U9" s="6"/>
-      <c r="V9" s="2"/>
-      <c r="W9" s="2"/>
+      <c r="T9" s="2"/>
+      <c r="U9" s="2"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="6"/>
       <c r="X9" s="2"/>
       <c r="Y9" s="2"/>
       <c r="Z9" s="2"/>
@@ -3034,10 +2834,10 @@
       <c r="AC9" s="2"/>
       <c r="AD9" s="2"/>
       <c r="AE9" s="2"/>
-      <c r="AF9" s="3"/>
-      <c r="AG9" s="6"/>
-      <c r="AH9" s="2"/>
-      <c r="AI9" s="2"/>
+      <c r="AF9" s="2"/>
+      <c r="AG9" s="2"/>
+      <c r="AH9" s="3"/>
+      <c r="AI9" s="6"/>
       <c r="AJ9" s="2"/>
       <c r="AK9" s="2"/>
       <c r="AL9" s="2"/>
@@ -3046,9 +2846,11 @@
       <c r="AO9" s="2"/>
       <c r="AP9" s="2"/>
       <c r="AQ9" s="2"/>
-      <c r="AR9" s="3"/>
+      <c r="AR9" s="2"/>
+      <c r="AS9" s="2"/>
+      <c r="AT9" s="3"/>
     </row>
-    <row r="10" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>46118</v>
       </c>
@@ -3057,11 +2859,14 @@
       <c r="D10" s="4"/>
       <c r="E10" s="2"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
+      <c r="G10" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="6"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
@@ -3070,10 +2875,10 @@
       <c r="Q10" s="2"/>
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
-      <c r="T10" s="3"/>
-      <c r="U10" s="6"/>
-      <c r="V10" s="2"/>
-      <c r="W10" s="2"/>
+      <c r="T10" s="2"/>
+      <c r="U10" s="2"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="6"/>
       <c r="X10" s="2"/>
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
@@ -3082,10 +2887,10 @@
       <c r="AC10" s="2"/>
       <c r="AD10" s="2"/>
       <c r="AE10" s="2"/>
-      <c r="AF10" s="3"/>
-      <c r="AG10" s="6"/>
-      <c r="AH10" s="2"/>
-      <c r="AI10" s="2"/>
+      <c r="AF10" s="2"/>
+      <c r="AG10" s="2"/>
+      <c r="AH10" s="3"/>
+      <c r="AI10" s="6"/>
       <c r="AJ10" s="2"/>
       <c r="AK10" s="2"/>
       <c r="AL10" s="2"/>
@@ -3094,9 +2899,11 @@
       <c r="AO10" s="2"/>
       <c r="AP10" s="2"/>
       <c r="AQ10" s="2"/>
-      <c r="AR10" s="3"/>
+      <c r="AR10" s="2"/>
+      <c r="AS10" s="2"/>
+      <c r="AT10" s="3"/>
     </row>
-    <row r="11" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7">
         <v>46119</v>
       </c>
@@ -3105,11 +2912,14 @@
       <c r="D11" s="4"/>
       <c r="E11" s="2"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
+      <c r="G11" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H11" s="3"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="6"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
@@ -3118,10 +2928,10 @@
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
-      <c r="T11" s="3"/>
-      <c r="U11" s="6"/>
-      <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="6"/>
       <c r="X11" s="2"/>
       <c r="Y11" s="2"/>
       <c r="Z11" s="2"/>
@@ -3130,10 +2940,10 @@
       <c r="AC11" s="2"/>
       <c r="AD11" s="2"/>
       <c r="AE11" s="2"/>
-      <c r="AF11" s="3"/>
-      <c r="AG11" s="6"/>
-      <c r="AH11" s="2"/>
-      <c r="AI11" s="2"/>
+      <c r="AF11" s="2"/>
+      <c r="AG11" s="2"/>
+      <c r="AH11" s="3"/>
+      <c r="AI11" s="6"/>
       <c r="AJ11" s="2"/>
       <c r="AK11" s="2"/>
       <c r="AL11" s="2"/>
@@ -3142,9 +2952,11 @@
       <c r="AO11" s="2"/>
       <c r="AP11" s="2"/>
       <c r="AQ11" s="2"/>
-      <c r="AR11" s="3"/>
+      <c r="AR11" s="2"/>
+      <c r="AS11" s="2"/>
+      <c r="AT11" s="3"/>
     </row>
-    <row r="12" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
         <v>46120</v>
       </c>
@@ -3153,11 +2965,14 @@
       <c r="D12" s="4"/>
       <c r="E12" s="2"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
+      <c r="G12" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="6"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
@@ -3166,10 +2981,10 @@
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
-      <c r="T12" s="3"/>
-      <c r="U12" s="6"/>
-      <c r="V12" s="2"/>
-      <c r="W12" s="2"/>
+      <c r="T12" s="2"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="6"/>
       <c r="X12" s="2"/>
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
@@ -3178,10 +2993,10 @@
       <c r="AC12" s="2"/>
       <c r="AD12" s="2"/>
       <c r="AE12" s="2"/>
-      <c r="AF12" s="3"/>
-      <c r="AG12" s="6"/>
-      <c r="AH12" s="2"/>
-      <c r="AI12" s="2"/>
+      <c r="AF12" s="2"/>
+      <c r="AG12" s="2"/>
+      <c r="AH12" s="3"/>
+      <c r="AI12" s="6"/>
       <c r="AJ12" s="2"/>
       <c r="AK12" s="2"/>
       <c r="AL12" s="2"/>
@@ -3190,9 +3005,11 @@
       <c r="AO12" s="2"/>
       <c r="AP12" s="2"/>
       <c r="AQ12" s="2"/>
-      <c r="AR12" s="3"/>
+      <c r="AR12" s="2"/>
+      <c r="AS12" s="2"/>
+      <c r="AT12" s="3"/>
     </row>
-    <row r="13" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
         <v>46121</v>
       </c>
@@ -3201,11 +3018,14 @@
       <c r="D13" s="4"/>
       <c r="E13" s="2"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
+      <c r="G13" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="6"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
@@ -3214,10 +3034,10 @@
       <c r="Q13" s="2"/>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
-      <c r="T13" s="3"/>
-      <c r="U13" s="6"/>
-      <c r="V13" s="2"/>
-      <c r="W13" s="2"/>
+      <c r="T13" s="2"/>
+      <c r="U13" s="2"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="6"/>
       <c r="X13" s="2"/>
       <c r="Y13" s="2"/>
       <c r="Z13" s="2"/>
@@ -3226,10 +3046,10 @@
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
       <c r="AE13" s="2"/>
-      <c r="AF13" s="3"/>
-      <c r="AG13" s="6"/>
-      <c r="AH13" s="2"/>
-      <c r="AI13" s="2"/>
+      <c r="AF13" s="2"/>
+      <c r="AG13" s="2"/>
+      <c r="AH13" s="3"/>
+      <c r="AI13" s="6"/>
       <c r="AJ13" s="2"/>
       <c r="AK13" s="2"/>
       <c r="AL13" s="2"/>
@@ -3238,9 +3058,11 @@
       <c r="AO13" s="2"/>
       <c r="AP13" s="2"/>
       <c r="AQ13" s="2"/>
-      <c r="AR13" s="3"/>
+      <c r="AR13" s="2"/>
+      <c r="AS13" s="2"/>
+      <c r="AT13" s="3"/>
     </row>
-    <row r="14" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7">
         <v>46122</v>
       </c>
@@ -3249,11 +3071,14 @@
       <c r="D14" s="4"/>
       <c r="E14" s="2"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
+      <c r="G14" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="6"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
@@ -3262,10 +3087,10 @@
       <c r="Q14" s="2"/>
       <c r="R14" s="2"/>
       <c r="S14" s="2"/>
-      <c r="T14" s="3"/>
-      <c r="U14" s="6"/>
-      <c r="V14" s="2"/>
-      <c r="W14" s="2"/>
+      <c r="T14" s="2"/>
+      <c r="U14" s="2"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="6"/>
       <c r="X14" s="2"/>
       <c r="Y14" s="2"/>
       <c r="Z14" s="2"/>
@@ -3274,10 +3099,10 @@
       <c r="AC14" s="2"/>
       <c r="AD14" s="2"/>
       <c r="AE14" s="2"/>
-      <c r="AF14" s="3"/>
-      <c r="AG14" s="6"/>
-      <c r="AH14" s="2"/>
-      <c r="AI14" s="2"/>
+      <c r="AF14" s="2"/>
+      <c r="AG14" s="2"/>
+      <c r="AH14" s="3"/>
+      <c r="AI14" s="6"/>
       <c r="AJ14" s="2"/>
       <c r="AK14" s="2"/>
       <c r="AL14" s="2"/>
@@ -3286,9 +3111,11 @@
       <c r="AO14" s="2"/>
       <c r="AP14" s="2"/>
       <c r="AQ14" s="2"/>
-      <c r="AR14" s="3"/>
+      <c r="AR14" s="2"/>
+      <c r="AS14" s="2"/>
+      <c r="AT14" s="3"/>
     </row>
-    <row r="15" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
         <v>46123</v>
       </c>
@@ -3297,11 +3124,14 @@
       <c r="D15" s="4"/>
       <c r="E15" s="2"/>
       <c r="F15" s="3"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
+      <c r="G15" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H15" s="3"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="6"/>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
@@ -3310,10 +3140,10 @@
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
-      <c r="T15" s="3"/>
-      <c r="U15" s="6"/>
-      <c r="V15" s="2"/>
-      <c r="W15" s="2"/>
+      <c r="T15" s="2"/>
+      <c r="U15" s="2"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="6"/>
       <c r="X15" s="2"/>
       <c r="Y15" s="2"/>
       <c r="Z15" s="2"/>
@@ -3322,10 +3152,10 @@
       <c r="AC15" s="2"/>
       <c r="AD15" s="2"/>
       <c r="AE15" s="2"/>
-      <c r="AF15" s="3"/>
-      <c r="AG15" s="6"/>
-      <c r="AH15" s="2"/>
-      <c r="AI15" s="2"/>
+      <c r="AF15" s="2"/>
+      <c r="AG15" s="2"/>
+      <c r="AH15" s="3"/>
+      <c r="AI15" s="6"/>
       <c r="AJ15" s="2"/>
       <c r="AK15" s="2"/>
       <c r="AL15" s="2"/>
@@ -3334,9 +3164,11 @@
       <c r="AO15" s="2"/>
       <c r="AP15" s="2"/>
       <c r="AQ15" s="2"/>
-      <c r="AR15" s="3"/>
+      <c r="AR15" s="2"/>
+      <c r="AS15" s="2"/>
+      <c r="AT15" s="3"/>
     </row>
-    <row r="16" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7">
         <v>46124</v>
       </c>
@@ -3345,11 +3177,14 @@
       <c r="D16" s="4"/>
       <c r="E16" s="2"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
+      <c r="G16" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="6"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
@@ -3358,10 +3193,10 @@
       <c r="Q16" s="2"/>
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
-      <c r="T16" s="3"/>
-      <c r="U16" s="6"/>
-      <c r="V16" s="2"/>
-      <c r="W16" s="2"/>
+      <c r="T16" s="2"/>
+      <c r="U16" s="2"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="6"/>
       <c r="X16" s="2"/>
       <c r="Y16" s="2"/>
       <c r="Z16" s="2"/>
@@ -3370,10 +3205,10 @@
       <c r="AC16" s="2"/>
       <c r="AD16" s="2"/>
       <c r="AE16" s="2"/>
-      <c r="AF16" s="3"/>
-      <c r="AG16" s="6"/>
-      <c r="AH16" s="2"/>
-      <c r="AI16" s="2"/>
+      <c r="AF16" s="2"/>
+      <c r="AG16" s="2"/>
+      <c r="AH16" s="3"/>
+      <c r="AI16" s="6"/>
       <c r="AJ16" s="2"/>
       <c r="AK16" s="2"/>
       <c r="AL16" s="2"/>
@@ -3382,9 +3217,11 @@
       <c r="AO16" s="2"/>
       <c r="AP16" s="2"/>
       <c r="AQ16" s="2"/>
-      <c r="AR16" s="3"/>
+      <c r="AR16" s="2"/>
+      <c r="AS16" s="2"/>
+      <c r="AT16" s="3"/>
     </row>
-    <row r="17" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
         <v>46125</v>
       </c>
@@ -3393,11 +3230,14 @@
       <c r="D17" s="4"/>
       <c r="E17" s="2"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
+      <c r="G17" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H17" s="3"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="6"/>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
@@ -3406,10 +3246,10 @@
       <c r="Q17" s="2"/>
       <c r="R17" s="2"/>
       <c r="S17" s="2"/>
-      <c r="T17" s="3"/>
-      <c r="U17" s="6"/>
-      <c r="V17" s="2"/>
-      <c r="W17" s="2"/>
+      <c r="T17" s="2"/>
+      <c r="U17" s="2"/>
+      <c r="V17" s="3"/>
+      <c r="W17" s="6"/>
       <c r="X17" s="2"/>
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
@@ -3418,10 +3258,10 @@
       <c r="AC17" s="2"/>
       <c r="AD17" s="2"/>
       <c r="AE17" s="2"/>
-      <c r="AF17" s="3"/>
-      <c r="AG17" s="6"/>
-      <c r="AH17" s="2"/>
-      <c r="AI17" s="2"/>
+      <c r="AF17" s="2"/>
+      <c r="AG17" s="2"/>
+      <c r="AH17" s="3"/>
+      <c r="AI17" s="6"/>
       <c r="AJ17" s="2"/>
       <c r="AK17" s="2"/>
       <c r="AL17" s="2"/>
@@ -3430,9 +3270,11 @@
       <c r="AO17" s="2"/>
       <c r="AP17" s="2"/>
       <c r="AQ17" s="2"/>
-      <c r="AR17" s="3"/>
+      <c r="AR17" s="2"/>
+      <c r="AS17" s="2"/>
+      <c r="AT17" s="3"/>
     </row>
-    <row r="18" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7">
         <v>46126</v>
       </c>
@@ -3441,11 +3283,14 @@
       <c r="D18" s="4"/>
       <c r="E18" s="2"/>
       <c r="F18" s="3"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
+      <c r="G18" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H18" s="3"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="6"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
@@ -3454,10 +3299,10 @@
       <c r="Q18" s="2"/>
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
-      <c r="T18" s="3"/>
-      <c r="U18" s="6"/>
-      <c r="V18" s="2"/>
-      <c r="W18" s="2"/>
+      <c r="T18" s="2"/>
+      <c r="U18" s="2"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="6"/>
       <c r="X18" s="2"/>
       <c r="Y18" s="2"/>
       <c r="Z18" s="2"/>
@@ -3466,10 +3311,10 @@
       <c r="AC18" s="2"/>
       <c r="AD18" s="2"/>
       <c r="AE18" s="2"/>
-      <c r="AF18" s="3"/>
-      <c r="AG18" s="6"/>
-      <c r="AH18" s="2"/>
-      <c r="AI18" s="2"/>
+      <c r="AF18" s="2"/>
+      <c r="AG18" s="2"/>
+      <c r="AH18" s="3"/>
+      <c r="AI18" s="6"/>
       <c r="AJ18" s="2"/>
       <c r="AK18" s="2"/>
       <c r="AL18" s="2"/>
@@ -3478,9 +3323,11 @@
       <c r="AO18" s="2"/>
       <c r="AP18" s="2"/>
       <c r="AQ18" s="2"/>
-      <c r="AR18" s="3"/>
+      <c r="AR18" s="2"/>
+      <c r="AS18" s="2"/>
+      <c r="AT18" s="3"/>
     </row>
-    <row r="19" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7">
         <v>46127</v>
       </c>
@@ -3489,11 +3336,14 @@
       <c r="D19" s="4"/>
       <c r="E19" s="2"/>
       <c r="F19" s="3"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
+      <c r="G19" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H19" s="3"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="6"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
@@ -3502,10 +3352,10 @@
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
       <c r="S19" s="2"/>
-      <c r="T19" s="3"/>
-      <c r="U19" s="6"/>
-      <c r="V19" s="2"/>
-      <c r="W19" s="2"/>
+      <c r="T19" s="2"/>
+      <c r="U19" s="2"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="6"/>
       <c r="X19" s="2"/>
       <c r="Y19" s="2"/>
       <c r="Z19" s="2"/>
@@ -3514,10 +3364,10 @@
       <c r="AC19" s="2"/>
       <c r="AD19" s="2"/>
       <c r="AE19" s="2"/>
-      <c r="AF19" s="3"/>
-      <c r="AG19" s="6"/>
-      <c r="AH19" s="2"/>
-      <c r="AI19" s="2"/>
+      <c r="AF19" s="2"/>
+      <c r="AG19" s="2"/>
+      <c r="AH19" s="3"/>
+      <c r="AI19" s="6"/>
       <c r="AJ19" s="2"/>
       <c r="AK19" s="2"/>
       <c r="AL19" s="2"/>
@@ -3526,9 +3376,11 @@
       <c r="AO19" s="2"/>
       <c r="AP19" s="2"/>
       <c r="AQ19" s="2"/>
-      <c r="AR19" s="3"/>
+      <c r="AR19" s="2"/>
+      <c r="AS19" s="2"/>
+      <c r="AT19" s="3"/>
     </row>
-    <row r="20" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7">
         <v>46128</v>
       </c>
@@ -3537,11 +3389,14 @@
       <c r="D20" s="4"/>
       <c r="E20" s="2"/>
       <c r="F20" s="3"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
+      <c r="G20" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H20" s="3"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="6"/>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
@@ -3550,10 +3405,10 @@
       <c r="Q20" s="2"/>
       <c r="R20" s="2"/>
       <c r="S20" s="2"/>
-      <c r="T20" s="3"/>
-      <c r="U20" s="6"/>
-      <c r="V20" s="2"/>
-      <c r="W20" s="2"/>
+      <c r="T20" s="2"/>
+      <c r="U20" s="2"/>
+      <c r="V20" s="3"/>
+      <c r="W20" s="6"/>
       <c r="X20" s="2"/>
       <c r="Y20" s="2"/>
       <c r="Z20" s="2"/>
@@ -3562,10 +3417,10 @@
       <c r="AC20" s="2"/>
       <c r="AD20" s="2"/>
       <c r="AE20" s="2"/>
-      <c r="AF20" s="3"/>
-      <c r="AG20" s="6"/>
-      <c r="AH20" s="2"/>
-      <c r="AI20" s="2"/>
+      <c r="AF20" s="2"/>
+      <c r="AG20" s="2"/>
+      <c r="AH20" s="3"/>
+      <c r="AI20" s="6"/>
       <c r="AJ20" s="2"/>
       <c r="AK20" s="2"/>
       <c r="AL20" s="2"/>
@@ -3574,9 +3429,11 @@
       <c r="AO20" s="2"/>
       <c r="AP20" s="2"/>
       <c r="AQ20" s="2"/>
-      <c r="AR20" s="3"/>
+      <c r="AR20" s="2"/>
+      <c r="AS20" s="2"/>
+      <c r="AT20" s="3"/>
     </row>
-    <row r="21" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7">
         <v>46129</v>
       </c>
@@ -3585,11 +3442,14 @@
       <c r="D21" s="4"/>
       <c r="E21" s="2"/>
       <c r="F21" s="3"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
+      <c r="G21" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H21" s="3"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="6"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
@@ -3598,10 +3458,10 @@
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
-      <c r="T21" s="3"/>
-      <c r="U21" s="6"/>
-      <c r="V21" s="2"/>
-      <c r="W21" s="2"/>
+      <c r="T21" s="2"/>
+      <c r="U21" s="2"/>
+      <c r="V21" s="3"/>
+      <c r="W21" s="6"/>
       <c r="X21" s="2"/>
       <c r="Y21" s="2"/>
       <c r="Z21" s="2"/>
@@ -3610,10 +3470,10 @@
       <c r="AC21" s="2"/>
       <c r="AD21" s="2"/>
       <c r="AE21" s="2"/>
-      <c r="AF21" s="3"/>
-      <c r="AG21" s="6"/>
-      <c r="AH21" s="2"/>
-      <c r="AI21" s="2"/>
+      <c r="AF21" s="2"/>
+      <c r="AG21" s="2"/>
+      <c r="AH21" s="3"/>
+      <c r="AI21" s="6"/>
       <c r="AJ21" s="2"/>
       <c r="AK21" s="2"/>
       <c r="AL21" s="2"/>
@@ -3622,9 +3482,11 @@
       <c r="AO21" s="2"/>
       <c r="AP21" s="2"/>
       <c r="AQ21" s="2"/>
-      <c r="AR21" s="3"/>
+      <c r="AR21" s="2"/>
+      <c r="AS21" s="2"/>
+      <c r="AT21" s="3"/>
     </row>
-    <row r="22" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
         <v>46130</v>
       </c>
@@ -3633,11 +3495,14 @@
       <c r="D22" s="4"/>
       <c r="E22" s="2"/>
       <c r="F22" s="3"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
+      <c r="G22" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H22" s="3"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="6"/>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
@@ -3646,10 +3511,10 @@
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
       <c r="S22" s="2"/>
-      <c r="T22" s="3"/>
-      <c r="U22" s="6"/>
-      <c r="V22" s="2"/>
-      <c r="W22" s="2"/>
+      <c r="T22" s="2"/>
+      <c r="U22" s="2"/>
+      <c r="V22" s="3"/>
+      <c r="W22" s="6"/>
       <c r="X22" s="2"/>
       <c r="Y22" s="2"/>
       <c r="Z22" s="2"/>
@@ -3658,11 +3523,11 @@
       <c r="AC22" s="2"/>
       <c r="AD22" s="2"/>
       <c r="AE22" s="2"/>
-      <c r="AF22" s="3"/>
-      <c r="AG22" s="6"/>
-      <c r="AH22" s="4"/>
-      <c r="AI22" s="2"/>
-      <c r="AJ22" s="2"/>
+      <c r="AF22" s="2"/>
+      <c r="AG22" s="2"/>
+      <c r="AH22" s="3"/>
+      <c r="AI22" s="6"/>
+      <c r="AJ22" s="4"/>
       <c r="AK22" s="2"/>
       <c r="AL22" s="2"/>
       <c r="AM22" s="2"/>
@@ -3671,8 +3536,10 @@
       <c r="AP22" s="2"/>
       <c r="AQ22" s="2"/>
       <c r="AR22" s="2"/>
+      <c r="AS22" s="2"/>
+      <c r="AT22" s="2"/>
     </row>
-    <row r="23" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7">
         <v>46131</v>
       </c>
@@ -3681,11 +3548,14 @@
       <c r="D23" s="4"/>
       <c r="E23" s="2"/>
       <c r="F23" s="3"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
+      <c r="G23" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H23" s="3"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="6"/>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
@@ -3694,10 +3564,10 @@
       <c r="Q23" s="2"/>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
-      <c r="T23" s="3"/>
-      <c r="U23" s="6"/>
-      <c r="V23" s="2"/>
-      <c r="W23" s="2"/>
+      <c r="T23" s="2"/>
+      <c r="U23" s="2"/>
+      <c r="V23" s="3"/>
+      <c r="W23" s="6"/>
       <c r="X23" s="2"/>
       <c r="Y23" s="2"/>
       <c r="Z23" s="2"/>
@@ -3706,11 +3576,11 @@
       <c r="AC23" s="2"/>
       <c r="AD23" s="2"/>
       <c r="AE23" s="2"/>
-      <c r="AF23" s="3"/>
-      <c r="AG23" s="6"/>
-      <c r="AH23" s="4"/>
-      <c r="AI23" s="2"/>
-      <c r="AJ23" s="2"/>
+      <c r="AF23" s="2"/>
+      <c r="AG23" s="2"/>
+      <c r="AH23" s="3"/>
+      <c r="AI23" s="6"/>
+      <c r="AJ23" s="4"/>
       <c r="AK23" s="2"/>
       <c r="AL23" s="2"/>
       <c r="AM23" s="2"/>
@@ -3719,8 +3589,10 @@
       <c r="AP23" s="2"/>
       <c r="AQ23" s="2"/>
       <c r="AR23" s="2"/>
+      <c r="AS23" s="2"/>
+      <c r="AT23" s="2"/>
     </row>
-    <row r="24" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
         <v>46132</v>
       </c>
@@ -3729,11 +3601,14 @@
       <c r="D24" s="4"/>
       <c r="E24" s="2"/>
       <c r="F24" s="3"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
+      <c r="G24" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H24" s="3"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="6"/>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
@@ -3742,10 +3617,10 @@
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
-      <c r="T24" s="3"/>
-      <c r="U24" s="6"/>
-      <c r="V24" s="2"/>
-      <c r="W24" s="2"/>
+      <c r="T24" s="2"/>
+      <c r="U24" s="2"/>
+      <c r="V24" s="3"/>
+      <c r="W24" s="6"/>
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
       <c r="Z24" s="2"/>
@@ -3754,11 +3629,11 @@
       <c r="AC24" s="2"/>
       <c r="AD24" s="2"/>
       <c r="AE24" s="2"/>
-      <c r="AF24" s="3"/>
-      <c r="AG24" s="6"/>
-      <c r="AH24" s="4"/>
-      <c r="AI24" s="2"/>
-      <c r="AJ24" s="2"/>
+      <c r="AF24" s="2"/>
+      <c r="AG24" s="2"/>
+      <c r="AH24" s="3"/>
+      <c r="AI24" s="6"/>
+      <c r="AJ24" s="4"/>
       <c r="AK24" s="2"/>
       <c r="AL24" s="2"/>
       <c r="AM24" s="2"/>
@@ -3767,8 +3642,10 @@
       <c r="AP24" s="2"/>
       <c r="AQ24" s="2"/>
       <c r="AR24" s="2"/>
+      <c r="AS24" s="2"/>
+      <c r="AT24" s="2"/>
     </row>
-    <row r="25" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7">
         <v>46133</v>
       </c>
@@ -3777,11 +3654,14 @@
       <c r="D25" s="4"/>
       <c r="E25" s="2"/>
       <c r="F25" s="3"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
+      <c r="G25" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H25" s="3"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="6"/>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
@@ -3790,10 +3670,10 @@
       <c r="Q25" s="2"/>
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
-      <c r="T25" s="3"/>
-      <c r="U25" s="6"/>
-      <c r="V25" s="2"/>
-      <c r="W25" s="2"/>
+      <c r="T25" s="2"/>
+      <c r="U25" s="2"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="6"/>
       <c r="X25" s="2"/>
       <c r="Y25" s="2"/>
       <c r="Z25" s="2"/>
@@ -3802,11 +3682,11 @@
       <c r="AC25" s="2"/>
       <c r="AD25" s="2"/>
       <c r="AE25" s="2"/>
-      <c r="AF25" s="3"/>
-      <c r="AG25" s="6"/>
-      <c r="AH25" s="4"/>
-      <c r="AI25" s="2"/>
-      <c r="AJ25" s="2"/>
+      <c r="AF25" s="2"/>
+      <c r="AG25" s="2"/>
+      <c r="AH25" s="3"/>
+      <c r="AI25" s="6"/>
+      <c r="AJ25" s="4"/>
       <c r="AK25" s="2"/>
       <c r="AL25" s="2"/>
       <c r="AM25" s="2"/>
@@ -3815,8 +3695,10 @@
       <c r="AP25" s="2"/>
       <c r="AQ25" s="2"/>
       <c r="AR25" s="2"/>
+      <c r="AS25" s="2"/>
+      <c r="AT25" s="2"/>
     </row>
-    <row r="26" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
         <v>46134</v>
       </c>
@@ -3825,11 +3707,14 @@
       <c r="D26" s="4"/>
       <c r="E26" s="2"/>
       <c r="F26" s="3"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
+      <c r="G26" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H26" s="3"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="6"/>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
@@ -3838,10 +3723,10 @@
       <c r="Q26" s="2"/>
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
-      <c r="T26" s="3"/>
-      <c r="U26" s="6"/>
-      <c r="V26" s="2"/>
-      <c r="W26" s="2"/>
+      <c r="T26" s="2"/>
+      <c r="U26" s="2"/>
+      <c r="V26" s="3"/>
+      <c r="W26" s="6"/>
       <c r="X26" s="2"/>
       <c r="Y26" s="2"/>
       <c r="Z26" s="2"/>
@@ -3850,11 +3735,11 @@
       <c r="AC26" s="2"/>
       <c r="AD26" s="2"/>
       <c r="AE26" s="2"/>
-      <c r="AF26" s="3"/>
-      <c r="AG26" s="6"/>
-      <c r="AH26" s="4"/>
-      <c r="AI26" s="2"/>
-      <c r="AJ26" s="2"/>
+      <c r="AF26" s="2"/>
+      <c r="AG26" s="2"/>
+      <c r="AH26" s="3"/>
+      <c r="AI26" s="6"/>
+      <c r="AJ26" s="4"/>
       <c r="AK26" s="2"/>
       <c r="AL26" s="2"/>
       <c r="AM26" s="2"/>
@@ -3863,8 +3748,10 @@
       <c r="AP26" s="2"/>
       <c r="AQ26" s="2"/>
       <c r="AR26" s="2"/>
+      <c r="AS26" s="2"/>
+      <c r="AT26" s="2"/>
     </row>
-    <row r="27" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7">
         <v>46135</v>
       </c>
@@ -3873,11 +3760,14 @@
       <c r="D27" s="4"/>
       <c r="E27" s="2"/>
       <c r="F27" s="3"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
+      <c r="G27" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H27" s="3"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="6"/>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
@@ -3886,10 +3776,10 @@
       <c r="Q27" s="2"/>
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
-      <c r="T27" s="3"/>
-      <c r="U27" s="6"/>
-      <c r="V27" s="2"/>
-      <c r="W27" s="2"/>
+      <c r="T27" s="2"/>
+      <c r="U27" s="2"/>
+      <c r="V27" s="3"/>
+      <c r="W27" s="6"/>
       <c r="X27" s="2"/>
       <c r="Y27" s="2"/>
       <c r="Z27" s="2"/>
@@ -3898,11 +3788,11 @@
       <c r="AC27" s="2"/>
       <c r="AD27" s="2"/>
       <c r="AE27" s="2"/>
-      <c r="AF27" s="3"/>
-      <c r="AG27" s="6"/>
-      <c r="AH27" s="4"/>
-      <c r="AI27" s="2"/>
-      <c r="AJ27" s="2"/>
+      <c r="AF27" s="2"/>
+      <c r="AG27" s="2"/>
+      <c r="AH27" s="3"/>
+      <c r="AI27" s="6"/>
+      <c r="AJ27" s="4"/>
       <c r="AK27" s="2"/>
       <c r="AL27" s="2"/>
       <c r="AM27" s="2"/>
@@ -3911,8 +3801,10 @@
       <c r="AP27" s="2"/>
       <c r="AQ27" s="2"/>
       <c r="AR27" s="2"/>
+      <c r="AS27" s="2"/>
+      <c r="AT27" s="2"/>
     </row>
-    <row r="28" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
         <v>46136</v>
       </c>
@@ -3921,11 +3813,14 @@
       <c r="D28" s="4"/>
       <c r="E28" s="2"/>
       <c r="F28" s="3"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="6"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
+      <c r="G28" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H28" s="3"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="6"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
@@ -3934,10 +3829,10 @@
       <c r="Q28" s="2"/>
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
-      <c r="T28" s="3"/>
-      <c r="U28" s="6"/>
-      <c r="V28" s="2"/>
-      <c r="W28" s="2"/>
+      <c r="T28" s="2"/>
+      <c r="U28" s="2"/>
+      <c r="V28" s="3"/>
+      <c r="W28" s="6"/>
       <c r="X28" s="2"/>
       <c r="Y28" s="2"/>
       <c r="Z28" s="2"/>
@@ -3946,11 +3841,11 @@
       <c r="AC28" s="2"/>
       <c r="AD28" s="2"/>
       <c r="AE28" s="2"/>
-      <c r="AF28" s="3"/>
-      <c r="AG28" s="6"/>
-      <c r="AH28" s="4"/>
-      <c r="AI28" s="2"/>
-      <c r="AJ28" s="2"/>
+      <c r="AF28" s="2"/>
+      <c r="AG28" s="2"/>
+      <c r="AH28" s="3"/>
+      <c r="AI28" s="6"/>
+      <c r="AJ28" s="4"/>
       <c r="AK28" s="2"/>
       <c r="AL28" s="2"/>
       <c r="AM28" s="2"/>
@@ -3959,8 +3854,10 @@
       <c r="AP28" s="2"/>
       <c r="AQ28" s="2"/>
       <c r="AR28" s="2"/>
+      <c r="AS28" s="2"/>
+      <c r="AT28" s="2"/>
     </row>
-    <row r="29" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7">
         <v>46137</v>
       </c>
@@ -3969,11 +3866,14 @@
       <c r="D29" s="4"/>
       <c r="E29" s="2"/>
       <c r="F29" s="3"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="6"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
+      <c r="G29" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H29" s="3"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="6"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
@@ -3982,10 +3882,10 @@
       <c r="Q29" s="2"/>
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
-      <c r="T29" s="3"/>
-      <c r="U29" s="6"/>
-      <c r="V29" s="2"/>
-      <c r="W29" s="2"/>
+      <c r="T29" s="2"/>
+      <c r="U29" s="2"/>
+      <c r="V29" s="3"/>
+      <c r="W29" s="6"/>
       <c r="X29" s="2"/>
       <c r="Y29" s="2"/>
       <c r="Z29" s="2"/>
@@ -3994,11 +3894,11 @@
       <c r="AC29" s="2"/>
       <c r="AD29" s="2"/>
       <c r="AE29" s="2"/>
-      <c r="AF29" s="3"/>
-      <c r="AG29" s="6"/>
-      <c r="AH29" s="4"/>
-      <c r="AI29" s="2"/>
-      <c r="AJ29" s="2"/>
+      <c r="AF29" s="2"/>
+      <c r="AG29" s="2"/>
+      <c r="AH29" s="3"/>
+      <c r="AI29" s="6"/>
+      <c r="AJ29" s="4"/>
       <c r="AK29" s="2"/>
       <c r="AL29" s="2"/>
       <c r="AM29" s="2"/>
@@ -4007,8 +3907,10 @@
       <c r="AP29" s="2"/>
       <c r="AQ29" s="2"/>
       <c r="AR29" s="2"/>
+      <c r="AS29" s="2"/>
+      <c r="AT29" s="2"/>
     </row>
-    <row r="30" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
         <v>46138</v>
       </c>
@@ -4027,164 +3929,169 @@
       <c r="E30" s="2">
         <v>77.91</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="3"/>
+      <c r="G30" s="3">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>91.807485900009425</v>
+      </c>
+      <c r="H30" s="3">
         <f>[1]PR_Calc!$AA$111</f>
         <v>2585.0777272727278</v>
       </c>
-      <c r="G30" s="2">
+      <c r="I30" s="2">
         <f>[1]PR_Calc!AN$111</f>
         <v>2575.6800000000003</v>
       </c>
-      <c r="H30" s="5">
+      <c r="J30" s="5">
         <f>[1]PR_Calc!BA$111</f>
         <v>2630.3231818181821</v>
       </c>
-      <c r="I30" s="6">
+      <c r="K30" s="6">
         <f>[1]PR_Calc!O$111</f>
         <v>0.85822998958753727</v>
       </c>
-      <c r="J30" s="2">
+      <c r="L30" s="2">
         <f>[1]PR_Calc!P$111</f>
         <v>0.8569062313765915</v>
       </c>
-      <c r="K30" s="2">
+      <c r="M30" s="2">
         <f>[1]PR_Calc!Q$111</f>
         <v>0.85982296382707624</v>
       </c>
-      <c r="L30" s="2">
+      <c r="N30" s="2">
         <f>[1]PR_Calc!R$111</f>
         <v>0.85966671030294295</v>
       </c>
-      <c r="M30" s="2">
+      <c r="O30" s="2">
         <f>[1]PR_Calc!S$111</f>
         <v>0.85880359559820818</v>
       </c>
-      <c r="N30" s="2">
+      <c r="P30" s="2">
         <f>[1]PR_Calc!T$111</f>
         <v>0.85674997785245799</v>
       </c>
-      <c r="O30" s="2">
+      <c r="Q30" s="2">
         <f>[1]PR_Calc!U$111</f>
         <v>0.85532881484724654</v>
       </c>
-      <c r="P30" s="2">
+      <c r="R30" s="2">
         <f>[1]PR_Calc!V$111</f>
         <v>0.83395488557588593</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="S30" s="2">
         <f>[1]PR_Calc!W$111</f>
         <v>0.83188379849203453</v>
       </c>
-      <c r="R30" s="2">
+      <c r="T30" s="2">
         <f>[1]PR_Calc!X$111</f>
         <v>0.82917928614886016</v>
       </c>
-      <c r="S30" s="2">
+      <c r="U30" s="2">
         <f>[1]PR_Calc!Y$111</f>
         <v>0.83039631670328851</v>
       </c>
-      <c r="T30" s="2">
+      <c r="V30" s="2">
         <f>[1]PR_Calc!Z$111</f>
         <v>0.85632586114409648</v>
       </c>
-      <c r="U30" s="6">
+      <c r="W30" s="6">
         <f>[1]PR_Calc!AB$111</f>
         <v>0.88474827088900154</v>
       </c>
-      <c r="V30" s="2">
+      <c r="X30" s="2">
         <f>[1]PR_Calc!AC$111</f>
         <v>0.85369931380985831</v>
       </c>
-      <c r="W30" s="2">
+      <c r="Y30" s="2">
         <f>[1]PR_Calc!AD$111</f>
         <v>0.8526501830049642</v>
       </c>
-      <c r="X30" s="2">
+      <c r="Z30" s="2">
         <f>[1]PR_Calc!AE$111</f>
         <v>0.88508345418566814</v>
       </c>
-      <c r="Y30" s="2">
+      <c r="AA30" s="2">
         <f>[1]PR_Calc!AF$111</f>
         <v>0.88811569377644273</v>
       </c>
-      <c r="Z30" s="2">
+      <c r="AB30" s="2">
         <f>[1]PR_Calc!AG$111</f>
         <v>0.82170629151640495</v>
       </c>
-      <c r="AA30" s="2">
+      <c r="AC30" s="2">
         <f>[1]PR_Calc!AH$111</f>
         <v>0.85136295159186715</v>
       </c>
-      <c r="AB30" s="2">
+      <c r="AD30" s="2">
         <f>[1]PR_Calc!AI$111</f>
         <v>0.82036115248256303</v>
       </c>
-      <c r="AC30" s="2">
+      <c r="AE30" s="2">
         <f>[1]PR_Calc!AJ$111</f>
         <v>0.81996970990657769</v>
       </c>
-      <c r="AD30" s="2">
+      <c r="AF30" s="2">
         <f>[1]PR_Calc!AK$111</f>
         <v>0.84956231574233276</v>
       </c>
-      <c r="AE30" s="2">
+      <c r="AG30" s="2">
         <f>[1]PR_Calc!AL$111</f>
         <v>0.81830429967420215</v>
       </c>
-      <c r="AF30" s="2">
+      <c r="AH30" s="2">
         <f>[1]PR_Calc!AM$111</f>
         <v>0.81933628464725528</v>
       </c>
-      <c r="AG30" s="6">
+      <c r="AI30" s="6">
         <f>[1]PR_Calc!AO$111</f>
         <v>0.83918598181860449</v>
       </c>
-      <c r="AH30" s="4">
+      <c r="AJ30" s="4">
         <f>[1]PR_Calc!AP$111</f>
         <v>0.83783372564701741</v>
       </c>
-      <c r="AI30" s="2">
+      <c r="AK30" s="2">
         <f>[1]PR_Calc!AQ$111</f>
         <v>0.83652417230190146</v>
       </c>
-      <c r="AJ30" s="2">
+      <c r="AL30" s="2">
         <f>[1]PR_Calc!AR$111</f>
         <v>0.83746363448426697</v>
       </c>
-      <c r="AK30" s="2">
+      <c r="AM30" s="2">
         <f>[1]PR_Calc!AS$111</f>
         <v>0.83758462582593529</v>
       </c>
-      <c r="AL30" s="2">
+      <c r="AN30" s="2">
         <f>[1]PR_Calc!AT$111</f>
         <v>0.84009697544998896</v>
       </c>
-      <c r="AM30" s="2">
+      <c r="AO30" s="2">
         <f>[1]PR_Calc!AU$111</f>
         <v>0.84015908865212896</v>
       </c>
-      <c r="AN30" s="2">
+      <c r="AP30" s="2">
         <f>[1]PR_Calc!AV$111</f>
         <v>0.83466659935040544</v>
       </c>
-      <c r="AO30" s="2">
+      <c r="AQ30" s="2">
         <f>[1]PR_Calc!AW$111</f>
         <v>0.83826787104947442</v>
       </c>
-      <c r="AP30" s="2">
+      <c r="AR30" s="2">
         <f>[1]PR_Calc!AX$111</f>
         <v>0.83846003376859424</v>
       </c>
-      <c r="AQ30" s="2">
+      <c r="AS30" s="2">
         <f>[1]PR_Calc!AY$111</f>
         <v>0.83796895126417592</v>
       </c>
-      <c r="AR30" s="2">
+      <c r="AT30" s="2">
         <f>[1]PR_Calc!AZ$111</f>
         <v>0.90562317480697996</v>
       </c>
     </row>
-    <row r="31" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7">
         <v>46139</v>
       </c>
@@ -4193,11 +4100,14 @@
       <c r="D31" s="4"/>
       <c r="E31" s="2"/>
       <c r="F31" s="3"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="6"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
+      <c r="G31" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H31" s="3"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="6"/>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
@@ -4206,10 +4116,10 @@
       <c r="Q31" s="2"/>
       <c r="R31" s="2"/>
       <c r="S31" s="2"/>
-      <c r="T31" s="3"/>
-      <c r="U31" s="6"/>
-      <c r="V31" s="2"/>
-      <c r="W31" s="2"/>
+      <c r="T31" s="2"/>
+      <c r="U31" s="2"/>
+      <c r="V31" s="3"/>
+      <c r="W31" s="6"/>
       <c r="X31" s="2"/>
       <c r="Y31" s="2"/>
       <c r="Z31" s="2"/>
@@ -4218,11 +4128,11 @@
       <c r="AC31" s="2"/>
       <c r="AD31" s="2"/>
       <c r="AE31" s="2"/>
-      <c r="AF31" s="3"/>
-      <c r="AG31" s="6"/>
-      <c r="AH31" s="4"/>
-      <c r="AI31" s="2"/>
-      <c r="AJ31" s="2"/>
+      <c r="AF31" s="2"/>
+      <c r="AG31" s="2"/>
+      <c r="AH31" s="3"/>
+      <c r="AI31" s="6"/>
+      <c r="AJ31" s="4"/>
       <c r="AK31" s="2"/>
       <c r="AL31" s="2"/>
       <c r="AM31" s="2"/>
@@ -4231,8 +4141,10 @@
       <c r="AP31" s="2"/>
       <c r="AQ31" s="2"/>
       <c r="AR31" s="2"/>
+      <c r="AS31" s="2"/>
+      <c r="AT31" s="2"/>
     </row>
-    <row r="32" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7">
         <v>46140</v>
       </c>
@@ -4241,11 +4153,14 @@
       <c r="D32" s="4"/>
       <c r="E32" s="2"/>
       <c r="F32" s="3"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="6"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
+      <c r="G32" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H32" s="3"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="6"/>
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
@@ -4254,10 +4169,10 @@
       <c r="Q32" s="2"/>
       <c r="R32" s="2"/>
       <c r="S32" s="2"/>
-      <c r="T32" s="3"/>
-      <c r="U32" s="6"/>
-      <c r="V32" s="2"/>
-      <c r="W32" s="2"/>
+      <c r="T32" s="2"/>
+      <c r="U32" s="2"/>
+      <c r="V32" s="3"/>
+      <c r="W32" s="6"/>
       <c r="X32" s="2"/>
       <c r="Y32" s="2"/>
       <c r="Z32" s="2"/>
@@ -4266,11 +4181,11 @@
       <c r="AC32" s="2"/>
       <c r="AD32" s="2"/>
       <c r="AE32" s="2"/>
-      <c r="AF32" s="3"/>
-      <c r="AG32" s="6"/>
-      <c r="AH32" s="4"/>
-      <c r="AI32" s="2"/>
-      <c r="AJ32" s="2"/>
+      <c r="AF32" s="2"/>
+      <c r="AG32" s="2"/>
+      <c r="AH32" s="3"/>
+      <c r="AI32" s="6"/>
+      <c r="AJ32" s="4"/>
       <c r="AK32" s="2"/>
       <c r="AL32" s="2"/>
       <c r="AM32" s="2"/>
@@ -4279,8 +4194,10 @@
       <c r="AP32" s="2"/>
       <c r="AQ32" s="2"/>
       <c r="AR32" s="2"/>
+      <c r="AS32" s="2"/>
+      <c r="AT32" s="2"/>
     </row>
-    <row r="33" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7">
         <v>46141</v>
       </c>
@@ -4289,11 +4206,14 @@
       <c r="D33" s="4"/>
       <c r="E33" s="2"/>
       <c r="F33" s="3"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
+      <c r="G33" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H33" s="3"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="6"/>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
@@ -4302,10 +4222,10 @@
       <c r="Q33" s="2"/>
       <c r="R33" s="2"/>
       <c r="S33" s="2"/>
-      <c r="T33" s="3"/>
-      <c r="U33" s="6"/>
-      <c r="V33" s="2"/>
-      <c r="W33" s="2"/>
+      <c r="T33" s="2"/>
+      <c r="U33" s="2"/>
+      <c r="V33" s="3"/>
+      <c r="W33" s="6"/>
       <c r="X33" s="2"/>
       <c r="Y33" s="2"/>
       <c r="Z33" s="2"/>
@@ -4314,10 +4234,10 @@
       <c r="AC33" s="2"/>
       <c r="AD33" s="2"/>
       <c r="AE33" s="2"/>
-      <c r="AF33" s="3"/>
-      <c r="AG33" s="6"/>
-      <c r="AH33" s="2"/>
-      <c r="AI33" s="2"/>
+      <c r="AF33" s="2"/>
+      <c r="AG33" s="2"/>
+      <c r="AH33" s="3"/>
+      <c r="AI33" s="6"/>
       <c r="AJ33" s="2"/>
       <c r="AK33" s="2"/>
       <c r="AL33" s="2"/>
@@ -4326,9 +4246,11 @@
       <c r="AO33" s="2"/>
       <c r="AP33" s="2"/>
       <c r="AQ33" s="2"/>
-      <c r="AR33" s="3"/>
+      <c r="AR33" s="2"/>
+      <c r="AS33" s="2"/>
+      <c r="AT33" s="3"/>
     </row>
-    <row r="34" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:46" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="7">
         <v>46142</v>
       </c>
@@ -4337,11 +4259,14 @@
       <c r="D34" s="4"/>
       <c r="E34" s="2"/>
       <c r="F34" s="3"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
+      <c r="G34" s="3" t="e">
+        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H34" s="3"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="6"/>
       <c r="L34" s="2"/>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
@@ -4350,10 +4275,10 @@
       <c r="Q34" s="2"/>
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
-      <c r="T34" s="3"/>
-      <c r="U34" s="6"/>
-      <c r="V34" s="2"/>
-      <c r="W34" s="2"/>
+      <c r="T34" s="2"/>
+      <c r="U34" s="2"/>
+      <c r="V34" s="3"/>
+      <c r="W34" s="6"/>
       <c r="X34" s="2"/>
       <c r="Y34" s="2"/>
       <c r="Z34" s="2"/>
@@ -4362,10 +4287,10 @@
       <c r="AC34" s="2"/>
       <c r="AD34" s="2"/>
       <c r="AE34" s="2"/>
-      <c r="AF34" s="3"/>
-      <c r="AG34" s="6"/>
-      <c r="AH34" s="2"/>
-      <c r="AI34" s="2"/>
+      <c r="AF34" s="2"/>
+      <c r="AG34" s="2"/>
+      <c r="AH34" s="3"/>
+      <c r="AI34" s="6"/>
       <c r="AJ34" s="2"/>
       <c r="AK34" s="2"/>
       <c r="AL34" s="2"/>
@@ -4374,9 +4299,11 @@
       <c r="AO34" s="2"/>
       <c r="AP34" s="2"/>
       <c r="AQ34" s="2"/>
-      <c r="AR34" s="3"/>
+      <c r="AR34" s="2"/>
+      <c r="AS34" s="2"/>
+      <c r="AT34" s="3"/>
     </row>
-    <row r="35" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:46" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="11"/>
       <c r="C35" s="11"/>
       <c r="D35" s="19">
@@ -4387,12 +4314,18 @@
         <f>AVERAGE(E5:E34)</f>
         <v>77.91</v>
       </c>
-      <c r="F35" s="12"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="14"/>
-      <c r="J35" s="15"/>
-      <c r="K35" s="15"/>
+      <c r="F35" s="30" t="e">
+        <f>AVERAGE(F5:F34)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G35" s="30" t="e">
+        <f>SUMIF(G5:G34,"&lt;&gt;100")/COUNTIF(G5:G34,"&lt;&gt;100")</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H35" s="12"/>
+      <c r="I35" s="11"/>
+      <c r="J35" s="13"/>
+      <c r="K35" s="14"/>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
       <c r="N35" s="15"/>
@@ -4401,10 +4334,10 @@
       <c r="Q35" s="15"/>
       <c r="R35" s="15"/>
       <c r="S35" s="15"/>
-      <c r="T35" s="16"/>
-      <c r="U35" s="17"/>
-      <c r="V35" s="18"/>
-      <c r="W35" s="18"/>
+      <c r="T35" s="15"/>
+      <c r="U35" s="15"/>
+      <c r="V35" s="16"/>
+      <c r="W35" s="17"/>
       <c r="X35" s="18"/>
       <c r="Y35" s="18"/>
       <c r="Z35" s="18"/>
@@ -4414,9 +4347,9 @@
       <c r="AD35" s="18"/>
       <c r="AE35" s="18"/>
       <c r="AF35" s="18"/>
-      <c r="AG35" s="17"/>
+      <c r="AG35" s="18"/>
       <c r="AH35" s="18"/>
-      <c r="AI35" s="18"/>
+      <c r="AI35" s="17"/>
       <c r="AJ35" s="18"/>
       <c r="AK35" s="18"/>
       <c r="AL35" s="18"/>
@@ -4426,13 +4359,15 @@
       <c r="AP35" s="18"/>
       <c r="AQ35" s="18"/>
       <c r="AR35" s="18"/>
+      <c r="AS35" s="18"/>
+      <c r="AT35" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:AR1"/>
+    <mergeCell ref="A1:AT1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D5:E34">
-    <cfRule type="cellIs" dxfId="54" priority="1" operator="greaterThan">
+  <conditionalFormatting sqref="D5:G34">
+    <cfRule type="cellIs" dxfId="46" priority="1" operator="greaterThan">
       <formula>100</formula>
     </cfRule>
     <cfRule type="colorScale" priority="13">
@@ -4444,7 +4379,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:AR34">
+  <conditionalFormatting sqref="K5:AT34">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="num" val="0"/>

</xml_diff>

<commit_message>
Add programmatic columns insertion to sync_mother_file and update availability formula to addition-based format
</commit_message>
<xml_diff>
--- a/original_format/00 PR_recalculation_APRL.xlsx
+++ b/original_format/00 PR_recalculation_APRL.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\S01\get\2025.01 Mazara 01 A2A\03 - REPORT\Report\09 Testing\PR Calculation automation\original_format\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77932A00-71C1-4946-B344-78BF3E058507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F9B91A-6FF7-41F5-8D54-20ECC1716594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
     <author>Utente</author>
   </authors>
   <commentList>
-    <comment ref="V6" authorId="0" shapeId="0" xr:uid="{2FB631FE-7B5E-43DD-B31B-4C74D1CA6B64}">
+    <comment ref="T6" authorId="0" shapeId="0" xr:uid="{2FB631FE-7B5E-43DD-B31B-4C74D1CA6B64}">
       <text>
         <r>
           <rPr>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>Dati</t>
   </si>
@@ -214,13 +214,6 @@
   <si>
     <t>PR calculation every day</t>
   </si>
-  <si>
-    <t>PR VCOM</t>
-  </si>
-  <si>
-    <t>External Availability
-[%]</t>
-  </si>
 </sst>
 </file>
 
@@ -286,7 +279,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -565,26 +558,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -609,6 +587,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -628,570 +609,1033 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="91">
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
+  <dxfs count="88">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color auto="1"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color auto="1"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color auto="1"/>
         </left>
-        <right style="medium">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="medium">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-410]d\-mmm\-yy;@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
         <right style="thin">
           <color auto="1"/>
         </right>
@@ -1213,23 +1657,6 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <top style="thin">
           <color auto="1"/>
@@ -1567,196 +1994,6 @@
         <horizontal style="thin">
           <color auto="1"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -2153,62 +2390,56 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TabellaAPRL2026" displayName="TabellaAPRL2026" ref="A4:AT35" headerRowCount="0" totalsRowCount="1">
-  <tableColumns count="46">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Colonna1"/>
-    <tableColumn id="2" xr3:uid="{B14D2040-0C85-4ABB-B9F2-DB214B494F99}" name="Colonna4" dataDxfId="90" totalsRowDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{6146493F-E789-4F9A-A367-EE09E8A74459}" name="Colonna11" dataDxfId="89" totalsRowDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{50DD95C4-E191-4573-9275-92130C5D20B6}" name="Colonna12" totalsRowFunction="custom" dataDxfId="88" totalsRowDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TabellaAPRL2026" displayName="TabellaAPRL2026" ref="A4:AR35" headerRowCount="0" totalsRowCount="1">
+  <tableColumns count="44">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Colonna1" totalsRowDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{B14D2040-0C85-4ABB-B9F2-DB214B494F99}" name="Colonna4" dataDxfId="87" totalsRowDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{6146493F-E789-4F9A-A367-EE09E8A74459}" name="Colonna11" dataDxfId="86" totalsRowDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{50DD95C4-E191-4573-9275-92130C5D20B6}" name="Colonna12" totalsRowFunction="custom" dataDxfId="85" totalsRowDxfId="40">
       <totalsRowFormula>AVERAGE(D5:D34)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{811DB1BF-4766-44EA-92AC-DE12BBC5C210}" name="Colonna7" totalsRowFunction="custom" dataDxfId="87" totalsRowDxfId="41">
+    <tableColumn id="5" xr3:uid="{811DB1BF-4766-44EA-92AC-DE12BBC5C210}" name="Colonna7" totalsRowFunction="custom" dataDxfId="84" totalsRowDxfId="39">
       <totalsRowFormula>AVERAGE(E5:E34)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{FCEE7969-4D4B-407C-97A5-5796C7281693}" name="Colonna9" totalsRowFunction="custom" dataDxfId="45" totalsRowDxfId="40">
-      <totalsRowFormula>AVERAGE(F5:F34)</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="9" xr3:uid="{A4FE1C65-5D9A-47C5-8BF7-1183770FC023}" name="Colonna8" totalsRowFunction="custom" dataDxfId="47" totalsRowDxfId="39">
-      <totalsRowFormula>SUMIF(G5:G34,"&lt;&gt;100")/COUNTIF(G5:G34,"&lt;&gt;100")</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="6" xr3:uid="{5F7D80EF-8BAA-4131-9F02-2B47B9B4D5BA}" name="Colonna13" dataDxfId="86" totalsRowDxfId="38"/>
-    <tableColumn id="7" xr3:uid="{55D2D573-983E-4C5B-9C48-1BACCA393A88}" name="Colonna14" dataDxfId="85" totalsRowDxfId="37"/>
-    <tableColumn id="8" xr3:uid="{7F240FDF-A189-4AF5-8F29-DEEFB888A9A0}" name="Colonna15" dataDxfId="84" totalsRowDxfId="36"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Colonna24" dataDxfId="83" totalsRowDxfId="35"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Colonna31" dataDxfId="82" totalsRowDxfId="34"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Colonna32" dataDxfId="81" totalsRowDxfId="33"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Colonna33" dataDxfId="80" totalsRowDxfId="32"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colonna34" dataDxfId="79" totalsRowDxfId="31"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Colonna35" dataDxfId="78" totalsRowDxfId="30"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Colonna36" dataDxfId="77" totalsRowDxfId="29"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Colonna37" dataDxfId="76" totalsRowDxfId="28"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Colonna3" dataDxfId="75" totalsRowDxfId="27"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Colonna17" dataDxfId="74" totalsRowDxfId="26"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Colonna19" dataDxfId="73" totalsRowDxfId="25"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Colonna20" dataDxfId="72" totalsRowDxfId="24"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Colonna39" dataDxfId="71" totalsRowDxfId="23"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Colonna40" dataDxfId="70" totalsRowDxfId="22"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Colonna41" dataDxfId="69" totalsRowDxfId="21"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Colonna42" dataDxfId="68" totalsRowDxfId="20"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Colonna43" dataDxfId="67" totalsRowDxfId="19"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Colonna44" dataDxfId="66" totalsRowDxfId="18"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Colonna45" dataDxfId="65" totalsRowDxfId="17"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="Colonna46" dataDxfId="64" totalsRowDxfId="16"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="Colonna38" dataDxfId="63" totalsRowDxfId="15"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Colonna2" dataDxfId="62" totalsRowDxfId="14"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Colonna5" dataDxfId="61" totalsRowDxfId="13"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Colonna6" dataDxfId="60" totalsRowDxfId="12"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="Colonna54" dataDxfId="59" totalsRowDxfId="11"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="Colonna55" dataDxfId="58" totalsRowDxfId="10"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0000-000030000000}" name="Colonna56" dataDxfId="57" totalsRowDxfId="9"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0000-000031000000}" name="Colonna57" dataDxfId="56" totalsRowDxfId="8"/>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0000-000032000000}" name="Colonna58" dataDxfId="55" totalsRowDxfId="7"/>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0000-000033000000}" name="Colonna59" dataDxfId="54" totalsRowDxfId="6"/>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0000-000034000000}" name="Colonna60" dataDxfId="53" totalsRowDxfId="5"/>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0000-000035000000}" name="Colonna61" dataDxfId="52" totalsRowDxfId="4"/>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0000-000036000000}" name="Colonna50" dataDxfId="51" totalsRowDxfId="3"/>
-    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0000-000037000000}" name="Colonna51" dataDxfId="50" totalsRowDxfId="2"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0000-000038000000}" name="Colonna52" dataDxfId="49" totalsRowDxfId="1"/>
-    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0000-000039000000}" name="Colonna53" dataDxfId="48" totalsRowDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{5F7D80EF-8BAA-4131-9F02-2B47B9B4D5BA}" name="Colonna13" dataDxfId="83" totalsRowDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{55D2D573-983E-4C5B-9C48-1BACCA393A88}" name="Colonna14" dataDxfId="82" totalsRowDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{7F240FDF-A189-4AF5-8F29-DEEFB888A9A0}" name="Colonna15" dataDxfId="81" totalsRowDxfId="36"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Colonna24" dataDxfId="80" totalsRowDxfId="35"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Colonna31" dataDxfId="53" totalsRowDxfId="34"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Colonna32" dataDxfId="52" totalsRowDxfId="33"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Colonna33" dataDxfId="51" totalsRowDxfId="32"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colonna34" dataDxfId="50" totalsRowDxfId="31"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Colonna35" dataDxfId="49" totalsRowDxfId="30"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Colonna36" dataDxfId="48" totalsRowDxfId="29"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Colonna37" dataDxfId="47" totalsRowDxfId="28"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Colonna3" dataDxfId="46" totalsRowDxfId="27"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Colonna17" dataDxfId="45" totalsRowDxfId="26"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Colonna19" dataDxfId="44" totalsRowDxfId="25"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Colonna20" dataDxfId="79" totalsRowDxfId="24"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Colonna39" dataDxfId="78" totalsRowDxfId="23"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Colonna40" dataDxfId="77" totalsRowDxfId="22"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Colonna41" dataDxfId="76" totalsRowDxfId="21"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Colonna42" dataDxfId="75" totalsRowDxfId="20"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Colonna43" dataDxfId="74" totalsRowDxfId="19"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Colonna44" dataDxfId="73" totalsRowDxfId="18"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Colonna45" dataDxfId="72" totalsRowDxfId="17"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="Colonna46" dataDxfId="71" totalsRowDxfId="16"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="Colonna38" dataDxfId="70" totalsRowDxfId="15"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Colonna2" dataDxfId="69" totalsRowDxfId="14"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Colonna5" dataDxfId="68" totalsRowDxfId="13"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Colonna6" dataDxfId="67" totalsRowDxfId="12"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="Colonna54" dataDxfId="66" totalsRowDxfId="11"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="Colonna55" dataDxfId="65" totalsRowDxfId="10"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0000-000030000000}" name="Colonna56" dataDxfId="64" totalsRowDxfId="9"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0000-000031000000}" name="Colonna57" dataDxfId="63" totalsRowDxfId="8"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0000-000032000000}" name="Colonna58" dataDxfId="62" totalsRowDxfId="7"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0000-000033000000}" name="Colonna59" dataDxfId="61" totalsRowDxfId="6"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0000-000034000000}" name="Colonna60" dataDxfId="60" totalsRowDxfId="5"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0000-000035000000}" name="Colonna61" dataDxfId="59" totalsRowDxfId="4"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0000-000036000000}" name="Colonna50" dataDxfId="58" totalsRowDxfId="3"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0000-000037000000}" name="Colonna51" dataDxfId="57" totalsRowDxfId="2"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0000-000038000000}" name="Colonna52" dataDxfId="56" totalsRowDxfId="1"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0000-000039000000}" name="Colonna53" dataDxfId="55" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2390,218 +2621,207 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AT35"/>
+  <dimension ref="A1:AR35"/>
   <sheetFormatPr defaultColWidth="13.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:46" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:44" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="29"/>
-      <c r="S1" s="29"/>
-      <c r="T1" s="29"/>
-      <c r="U1" s="29"/>
-      <c r="V1" s="29"/>
-      <c r="W1" s="29"/>
-      <c r="X1" s="29"/>
-      <c r="Y1" s="29"/>
-      <c r="Z1" s="29"/>
-      <c r="AA1" s="29"/>
-      <c r="AB1" s="29"/>
-      <c r="AC1" s="29"/>
-      <c r="AD1" s="29"/>
-      <c r="AE1" s="29"/>
-      <c r="AF1" s="29"/>
-      <c r="AG1" s="29"/>
-      <c r="AH1" s="29"/>
-      <c r="AI1" s="29"/>
-      <c r="AJ1" s="29"/>
-      <c r="AK1" s="29"/>
-      <c r="AL1" s="29"/>
-      <c r="AM1" s="29"/>
-      <c r="AN1" s="29"/>
-      <c r="AO1" s="29"/>
-      <c r="AP1" s="29"/>
-      <c r="AQ1" s="29"/>
-      <c r="AR1" s="29"/>
-      <c r="AS1" s="29"/>
-      <c r="AT1" s="29"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+      <c r="T1" s="20"/>
+      <c r="U1" s="20"/>
+      <c r="V1" s="20"/>
+      <c r="W1" s="20"/>
+      <c r="X1" s="20"/>
+      <c r="Y1" s="20"/>
+      <c r="Z1" s="20"/>
+      <c r="AA1" s="20"/>
+      <c r="AB1" s="20"/>
+      <c r="AC1" s="20"/>
+      <c r="AD1" s="20"/>
+      <c r="AE1" s="20"/>
+      <c r="AF1" s="20"/>
+      <c r="AG1" s="20"/>
+      <c r="AH1" s="20"/>
+      <c r="AI1" s="20"/>
+      <c r="AJ1" s="20"/>
+      <c r="AK1" s="20"/>
+      <c r="AL1" s="20"/>
+      <c r="AM1" s="20"/>
+      <c r="AN1" s="20"/>
+      <c r="AO1" s="20"/>
+      <c r="AP1" s="20"/>
+      <c r="AQ1" s="20"/>
+      <c r="AR1" s="20"/>
     </row>
-    <row r="2" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:46" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:46" s="1" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:44" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:44" s="1" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>45</v>
+      <c r="F4" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="I4" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="J4" s="27" t="s">
+      <c r="H4" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="K4" s="28" t="s">
+      <c r="I4" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="L4" s="24" t="s">
+      <c r="J4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="24" t="s">
+      <c r="K4" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="24" t="s">
+      <c r="L4" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="O4" s="24" t="s">
+      <c r="M4" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="P4" s="24" t="s">
+      <c r="N4" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="24" t="s">
+      <c r="O4" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="24" t="s">
+      <c r="P4" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="S4" s="24" t="s">
+      <c r="Q4" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="T4" s="24" t="s">
+      <c r="R4" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="U4" s="24" t="s">
+      <c r="S4" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="V4" s="27" t="s">
+      <c r="T4" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="W4" s="28" t="s">
+      <c r="U4" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="X4" s="24" t="s">
+      <c r="V4" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="Y4" s="24" t="s">
+      <c r="W4" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="Z4" s="24" t="s">
+      <c r="X4" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="AA4" s="24" t="s">
+      <c r="Y4" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="AB4" s="24" t="s">
+      <c r="Z4" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="AC4" s="24" t="s">
+      <c r="AA4" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="AD4" s="24" t="s">
+      <c r="AB4" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="AE4" s="24" t="s">
+      <c r="AC4" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="AF4" s="24" t="s">
+      <c r="AD4" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="AG4" s="24" t="s">
+      <c r="AE4" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="AH4" s="27" t="s">
+      <c r="AF4" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="AI4" s="28" t="s">
+      <c r="AG4" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="AJ4" s="24" t="s">
+      <c r="AH4" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="AK4" s="24" t="s">
+      <c r="AI4" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="AL4" s="24" t="s">
+      <c r="AJ4" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="AM4" s="24" t="s">
+      <c r="AK4" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="AN4" s="24" t="s">
+      <c r="AL4" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="AO4" s="24" t="s">
+      <c r="AM4" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="AP4" s="24" t="s">
+      <c r="AN4" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="AQ4" s="24" t="s">
+      <c r="AO4" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="AR4" s="24" t="s">
+      <c r="AP4" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="AS4" s="24" t="s">
+      <c r="AQ4" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="AT4" s="27" t="s">
+      <c r="AR4" s="28" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
         <v>46113</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
-      <c r="D5" s="20"/>
+      <c r="D5" s="21"/>
       <c r="E5" s="10"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H5" s="21"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="23"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
       <c r="L5" s="10"/>
       <c r="M5" s="10"/>
       <c r="N5" s="10"/>
@@ -2610,10 +2830,10 @@
       <c r="Q5" s="10"/>
       <c r="R5" s="10"/>
       <c r="S5" s="10"/>
-      <c r="T5" s="10"/>
-      <c r="U5" s="10"/>
-      <c r="V5" s="21"/>
-      <c r="W5" s="23"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="24"/>
+      <c r="V5" s="10"/>
+      <c r="W5" s="10"/>
       <c r="X5" s="10"/>
       <c r="Y5" s="10"/>
       <c r="Z5" s="10"/>
@@ -2622,10 +2842,10 @@
       <c r="AC5" s="10"/>
       <c r="AD5" s="10"/>
       <c r="AE5" s="10"/>
-      <c r="AF5" s="10"/>
-      <c r="AG5" s="10"/>
-      <c r="AH5" s="21"/>
-      <c r="AI5" s="23"/>
+      <c r="AF5" s="22"/>
+      <c r="AG5" s="24"/>
+      <c r="AH5" s="10"/>
+      <c r="AI5" s="10"/>
       <c r="AJ5" s="10"/>
       <c r="AK5" s="10"/>
       <c r="AL5" s="10"/>
@@ -2634,11 +2854,9 @@
       <c r="AO5" s="10"/>
       <c r="AP5" s="10"/>
       <c r="AQ5" s="10"/>
-      <c r="AR5" s="10"/>
-      <c r="AS5" s="10"/>
-      <c r="AT5" s="21"/>
+      <c r="AR5" s="22"/>
     </row>
-    <row r="6" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>46114</v>
       </c>
@@ -2647,14 +2865,11 @@
       <c r="D6" s="4"/>
       <c r="E6" s="2"/>
       <c r="F6" s="3"/>
-      <c r="G6" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="6"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -2663,10 +2878,10 @@
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
-      <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="6"/>
+      <c r="T6" s="3"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
       <c r="X6" s="2"/>
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
@@ -2675,10 +2890,10 @@
       <c r="AC6" s="2"/>
       <c r="AD6" s="2"/>
       <c r="AE6" s="2"/>
-      <c r="AF6" s="2"/>
-      <c r="AG6" s="2"/>
-      <c r="AH6" s="3"/>
-      <c r="AI6" s="6"/>
+      <c r="AF6" s="3"/>
+      <c r="AG6" s="6"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
       <c r="AK6" s="2"/>
       <c r="AL6" s="2"/>
@@ -2687,11 +2902,9 @@
       <c r="AO6" s="2"/>
       <c r="AP6" s="2"/>
       <c r="AQ6" s="2"/>
-      <c r="AR6" s="2"/>
-      <c r="AS6" s="2"/>
-      <c r="AT6" s="3"/>
+      <c r="AR6" s="3"/>
     </row>
-    <row r="7" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>46115</v>
       </c>
@@ -2700,14 +2913,11 @@
       <c r="D7" s="4"/>
       <c r="E7" s="2"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H7" s="3"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="6"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -2716,10 +2926,10 @@
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
-      <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="6"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
       <c r="X7" s="2"/>
       <c r="Y7" s="2"/>
       <c r="Z7" s="2"/>
@@ -2728,10 +2938,10 @@
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
       <c r="AE7" s="2"/>
-      <c r="AF7" s="2"/>
-      <c r="AG7" s="2"/>
-      <c r="AH7" s="3"/>
-      <c r="AI7" s="6"/>
+      <c r="AF7" s="3"/>
+      <c r="AG7" s="6"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
       <c r="AK7" s="2"/>
       <c r="AL7" s="2"/>
@@ -2740,11 +2950,9 @@
       <c r="AO7" s="2"/>
       <c r="AP7" s="2"/>
       <c r="AQ7" s="2"/>
-      <c r="AR7" s="2"/>
-      <c r="AS7" s="2"/>
-      <c r="AT7" s="3"/>
+      <c r="AR7" s="3"/>
     </row>
-    <row r="8" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
         <v>46116</v>
       </c>
@@ -2753,14 +2961,11 @@
       <c r="D8" s="4"/>
       <c r="E8" s="2"/>
       <c r="F8" s="3"/>
-      <c r="G8" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H8" s="3"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="6"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
@@ -2769,10 +2974,10 @@
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="3"/>
-      <c r="W8" s="6"/>
+      <c r="T8" s="3"/>
+      <c r="U8" s="6"/>
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
       <c r="X8" s="2"/>
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
@@ -2781,10 +2986,10 @@
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
       <c r="AE8" s="2"/>
-      <c r="AF8" s="2"/>
-      <c r="AG8" s="2"/>
-      <c r="AH8" s="3"/>
-      <c r="AI8" s="6"/>
+      <c r="AF8" s="3"/>
+      <c r="AG8" s="6"/>
+      <c r="AH8" s="2"/>
+      <c r="AI8" s="2"/>
       <c r="AJ8" s="2"/>
       <c r="AK8" s="2"/>
       <c r="AL8" s="2"/>
@@ -2793,11 +2998,9 @@
       <c r="AO8" s="2"/>
       <c r="AP8" s="2"/>
       <c r="AQ8" s="2"/>
-      <c r="AR8" s="2"/>
-      <c r="AS8" s="2"/>
-      <c r="AT8" s="3"/>
+      <c r="AR8" s="3"/>
     </row>
-    <row r="9" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>46117</v>
       </c>
@@ -2806,14 +3009,11 @@
       <c r="D9" s="4"/>
       <c r="E9" s="2"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H9" s="3"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="6"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
@@ -2822,10 +3022,10 @@
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
       <c r="S9" s="2"/>
-      <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="3"/>
-      <c r="W9" s="6"/>
+      <c r="T9" s="3"/>
+      <c r="U9" s="6"/>
+      <c r="V9" s="2"/>
+      <c r="W9" s="2"/>
       <c r="X9" s="2"/>
       <c r="Y9" s="2"/>
       <c r="Z9" s="2"/>
@@ -2834,10 +3034,10 @@
       <c r="AC9" s="2"/>
       <c r="AD9" s="2"/>
       <c r="AE9" s="2"/>
-      <c r="AF9" s="2"/>
-      <c r="AG9" s="2"/>
-      <c r="AH9" s="3"/>
-      <c r="AI9" s="6"/>
+      <c r="AF9" s="3"/>
+      <c r="AG9" s="6"/>
+      <c r="AH9" s="2"/>
+      <c r="AI9" s="2"/>
       <c r="AJ9" s="2"/>
       <c r="AK9" s="2"/>
       <c r="AL9" s="2"/>
@@ -2846,11 +3046,9 @@
       <c r="AO9" s="2"/>
       <c r="AP9" s="2"/>
       <c r="AQ9" s="2"/>
-      <c r="AR9" s="2"/>
-      <c r="AS9" s="2"/>
-      <c r="AT9" s="3"/>
+      <c r="AR9" s="3"/>
     </row>
-    <row r="10" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>46118</v>
       </c>
@@ -2859,14 +3057,11 @@
       <c r="D10" s="4"/>
       <c r="E10" s="2"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H10" s="3"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="6"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
@@ -2875,10 +3070,10 @@
       <c r="Q10" s="2"/>
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
-      <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="6"/>
+      <c r="T10" s="3"/>
+      <c r="U10" s="6"/>
+      <c r="V10" s="2"/>
+      <c r="W10" s="2"/>
       <c r="X10" s="2"/>
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
@@ -2887,10 +3082,10 @@
       <c r="AC10" s="2"/>
       <c r="AD10" s="2"/>
       <c r="AE10" s="2"/>
-      <c r="AF10" s="2"/>
-      <c r="AG10" s="2"/>
-      <c r="AH10" s="3"/>
-      <c r="AI10" s="6"/>
+      <c r="AF10" s="3"/>
+      <c r="AG10" s="6"/>
+      <c r="AH10" s="2"/>
+      <c r="AI10" s="2"/>
       <c r="AJ10" s="2"/>
       <c r="AK10" s="2"/>
       <c r="AL10" s="2"/>
@@ -2899,11 +3094,9 @@
       <c r="AO10" s="2"/>
       <c r="AP10" s="2"/>
       <c r="AQ10" s="2"/>
-      <c r="AR10" s="2"/>
-      <c r="AS10" s="2"/>
-      <c r="AT10" s="3"/>
+      <c r="AR10" s="3"/>
     </row>
-    <row r="11" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7">
         <v>46119</v>
       </c>
@@ -2912,14 +3105,11 @@
       <c r="D11" s="4"/>
       <c r="E11" s="2"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H11" s="3"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="6"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
@@ -2928,10 +3118,10 @@
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
-      <c r="T11" s="2"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="3"/>
-      <c r="W11" s="6"/>
+      <c r="T11" s="3"/>
+      <c r="U11" s="6"/>
+      <c r="V11" s="2"/>
+      <c r="W11" s="2"/>
       <c r="X11" s="2"/>
       <c r="Y11" s="2"/>
       <c r="Z11" s="2"/>
@@ -2940,10 +3130,10 @@
       <c r="AC11" s="2"/>
       <c r="AD11" s="2"/>
       <c r="AE11" s="2"/>
-      <c r="AF11" s="2"/>
-      <c r="AG11" s="2"/>
-      <c r="AH11" s="3"/>
-      <c r="AI11" s="6"/>
+      <c r="AF11" s="3"/>
+      <c r="AG11" s="6"/>
+      <c r="AH11" s="2"/>
+      <c r="AI11" s="2"/>
       <c r="AJ11" s="2"/>
       <c r="AK11" s="2"/>
       <c r="AL11" s="2"/>
@@ -2952,11 +3142,9 @@
       <c r="AO11" s="2"/>
       <c r="AP11" s="2"/>
       <c r="AQ11" s="2"/>
-      <c r="AR11" s="2"/>
-      <c r="AS11" s="2"/>
-      <c r="AT11" s="3"/>
+      <c r="AR11" s="3"/>
     </row>
-    <row r="12" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
         <v>46120</v>
       </c>
@@ -2965,14 +3153,11 @@
       <c r="D12" s="4"/>
       <c r="E12" s="2"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H12" s="3"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="6"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
@@ -2981,10 +3166,10 @@
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
-      <c r="T12" s="2"/>
-      <c r="U12" s="2"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="6"/>
+      <c r="T12" s="3"/>
+      <c r="U12" s="6"/>
+      <c r="V12" s="2"/>
+      <c r="W12" s="2"/>
       <c r="X12" s="2"/>
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
@@ -2993,10 +3178,10 @@
       <c r="AC12" s="2"/>
       <c r="AD12" s="2"/>
       <c r="AE12" s="2"/>
-      <c r="AF12" s="2"/>
-      <c r="AG12" s="2"/>
-      <c r="AH12" s="3"/>
-      <c r="AI12" s="6"/>
+      <c r="AF12" s="3"/>
+      <c r="AG12" s="6"/>
+      <c r="AH12" s="2"/>
+      <c r="AI12" s="2"/>
       <c r="AJ12" s="2"/>
       <c r="AK12" s="2"/>
       <c r="AL12" s="2"/>
@@ -3005,11 +3190,9 @@
       <c r="AO12" s="2"/>
       <c r="AP12" s="2"/>
       <c r="AQ12" s="2"/>
-      <c r="AR12" s="2"/>
-      <c r="AS12" s="2"/>
-      <c r="AT12" s="3"/>
+      <c r="AR12" s="3"/>
     </row>
-    <row r="13" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
         <v>46121</v>
       </c>
@@ -3018,14 +3201,11 @@
       <c r="D13" s="4"/>
       <c r="E13" s="2"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H13" s="3"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="6"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
@@ -3034,10 +3214,10 @@
       <c r="Q13" s="2"/>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
-      <c r="T13" s="2"/>
-      <c r="U13" s="2"/>
-      <c r="V13" s="3"/>
-      <c r="W13" s="6"/>
+      <c r="T13" s="3"/>
+      <c r="U13" s="6"/>
+      <c r="V13" s="2"/>
+      <c r="W13" s="2"/>
       <c r="X13" s="2"/>
       <c r="Y13" s="2"/>
       <c r="Z13" s="2"/>
@@ -3046,10 +3226,10 @@
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
       <c r="AE13" s="2"/>
-      <c r="AF13" s="2"/>
-      <c r="AG13" s="2"/>
-      <c r="AH13" s="3"/>
-      <c r="AI13" s="6"/>
+      <c r="AF13" s="3"/>
+      <c r="AG13" s="6"/>
+      <c r="AH13" s="2"/>
+      <c r="AI13" s="2"/>
       <c r="AJ13" s="2"/>
       <c r="AK13" s="2"/>
       <c r="AL13" s="2"/>
@@ -3058,11 +3238,9 @@
       <c r="AO13" s="2"/>
       <c r="AP13" s="2"/>
       <c r="AQ13" s="2"/>
-      <c r="AR13" s="2"/>
-      <c r="AS13" s="2"/>
-      <c r="AT13" s="3"/>
+      <c r="AR13" s="3"/>
     </row>
-    <row r="14" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7">
         <v>46122</v>
       </c>
@@ -3071,14 +3249,11 @@
       <c r="D14" s="4"/>
       <c r="E14" s="2"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H14" s="3"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="6"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
@@ -3087,10 +3262,10 @@
       <c r="Q14" s="2"/>
       <c r="R14" s="2"/>
       <c r="S14" s="2"/>
-      <c r="T14" s="2"/>
-      <c r="U14" s="2"/>
-      <c r="V14" s="3"/>
-      <c r="W14" s="6"/>
+      <c r="T14" s="3"/>
+      <c r="U14" s="6"/>
+      <c r="V14" s="2"/>
+      <c r="W14" s="2"/>
       <c r="X14" s="2"/>
       <c r="Y14" s="2"/>
       <c r="Z14" s="2"/>
@@ -3099,10 +3274,10 @@
       <c r="AC14" s="2"/>
       <c r="AD14" s="2"/>
       <c r="AE14" s="2"/>
-      <c r="AF14" s="2"/>
-      <c r="AG14" s="2"/>
-      <c r="AH14" s="3"/>
-      <c r="AI14" s="6"/>
+      <c r="AF14" s="3"/>
+      <c r="AG14" s="6"/>
+      <c r="AH14" s="2"/>
+      <c r="AI14" s="2"/>
       <c r="AJ14" s="2"/>
       <c r="AK14" s="2"/>
       <c r="AL14" s="2"/>
@@ -3111,11 +3286,9 @@
       <c r="AO14" s="2"/>
       <c r="AP14" s="2"/>
       <c r="AQ14" s="2"/>
-      <c r="AR14" s="2"/>
-      <c r="AS14" s="2"/>
-      <c r="AT14" s="3"/>
+      <c r="AR14" s="3"/>
     </row>
-    <row r="15" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
         <v>46123</v>
       </c>
@@ -3124,14 +3297,11 @@
       <c r="D15" s="4"/>
       <c r="E15" s="2"/>
       <c r="F15" s="3"/>
-      <c r="G15" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H15" s="3"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="6"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
@@ -3140,10 +3310,10 @@
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
-      <c r="T15" s="2"/>
-      <c r="U15" s="2"/>
-      <c r="V15" s="3"/>
-      <c r="W15" s="6"/>
+      <c r="T15" s="3"/>
+      <c r="U15" s="6"/>
+      <c r="V15" s="2"/>
+      <c r="W15" s="2"/>
       <c r="X15" s="2"/>
       <c r="Y15" s="2"/>
       <c r="Z15" s="2"/>
@@ -3152,10 +3322,10 @@
       <c r="AC15" s="2"/>
       <c r="AD15" s="2"/>
       <c r="AE15" s="2"/>
-      <c r="AF15" s="2"/>
-      <c r="AG15" s="2"/>
-      <c r="AH15" s="3"/>
-      <c r="AI15" s="6"/>
+      <c r="AF15" s="3"/>
+      <c r="AG15" s="6"/>
+      <c r="AH15" s="2"/>
+      <c r="AI15" s="2"/>
       <c r="AJ15" s="2"/>
       <c r="AK15" s="2"/>
       <c r="AL15" s="2"/>
@@ -3164,11 +3334,9 @@
       <c r="AO15" s="2"/>
       <c r="AP15" s="2"/>
       <c r="AQ15" s="2"/>
-      <c r="AR15" s="2"/>
-      <c r="AS15" s="2"/>
-      <c r="AT15" s="3"/>
+      <c r="AR15" s="3"/>
     </row>
-    <row r="16" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7">
         <v>46124</v>
       </c>
@@ -3177,14 +3345,11 @@
       <c r="D16" s="4"/>
       <c r="E16" s="2"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H16" s="3"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="6"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
@@ -3193,10 +3358,10 @@
       <c r="Q16" s="2"/>
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
-      <c r="T16" s="2"/>
-      <c r="U16" s="2"/>
-      <c r="V16" s="3"/>
-      <c r="W16" s="6"/>
+      <c r="T16" s="3"/>
+      <c r="U16" s="6"/>
+      <c r="V16" s="2"/>
+      <c r="W16" s="2"/>
       <c r="X16" s="2"/>
       <c r="Y16" s="2"/>
       <c r="Z16" s="2"/>
@@ -3205,10 +3370,10 @@
       <c r="AC16" s="2"/>
       <c r="AD16" s="2"/>
       <c r="AE16" s="2"/>
-      <c r="AF16" s="2"/>
-      <c r="AG16" s="2"/>
-      <c r="AH16" s="3"/>
-      <c r="AI16" s="6"/>
+      <c r="AF16" s="3"/>
+      <c r="AG16" s="6"/>
+      <c r="AH16" s="2"/>
+      <c r="AI16" s="2"/>
       <c r="AJ16" s="2"/>
       <c r="AK16" s="2"/>
       <c r="AL16" s="2"/>
@@ -3217,11 +3382,9 @@
       <c r="AO16" s="2"/>
       <c r="AP16" s="2"/>
       <c r="AQ16" s="2"/>
-      <c r="AR16" s="2"/>
-      <c r="AS16" s="2"/>
-      <c r="AT16" s="3"/>
+      <c r="AR16" s="3"/>
     </row>
-    <row r="17" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
         <v>46125</v>
       </c>
@@ -3230,14 +3393,11 @@
       <c r="D17" s="4"/>
       <c r="E17" s="2"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H17" s="3"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="6"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
@@ -3246,10 +3406,10 @@
       <c r="Q17" s="2"/>
       <c r="R17" s="2"/>
       <c r="S17" s="2"/>
-      <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
-      <c r="V17" s="3"/>
-      <c r="W17" s="6"/>
+      <c r="T17" s="3"/>
+      <c r="U17" s="6"/>
+      <c r="V17" s="2"/>
+      <c r="W17" s="2"/>
       <c r="X17" s="2"/>
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
@@ -3258,10 +3418,10 @@
       <c r="AC17" s="2"/>
       <c r="AD17" s="2"/>
       <c r="AE17" s="2"/>
-      <c r="AF17" s="2"/>
-      <c r="AG17" s="2"/>
-      <c r="AH17" s="3"/>
-      <c r="AI17" s="6"/>
+      <c r="AF17" s="3"/>
+      <c r="AG17" s="6"/>
+      <c r="AH17" s="2"/>
+      <c r="AI17" s="2"/>
       <c r="AJ17" s="2"/>
       <c r="AK17" s="2"/>
       <c r="AL17" s="2"/>
@@ -3270,11 +3430,9 @@
       <c r="AO17" s="2"/>
       <c r="AP17" s="2"/>
       <c r="AQ17" s="2"/>
-      <c r="AR17" s="2"/>
-      <c r="AS17" s="2"/>
-      <c r="AT17" s="3"/>
+      <c r="AR17" s="3"/>
     </row>
-    <row r="18" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7">
         <v>46126</v>
       </c>
@@ -3283,14 +3441,11 @@
       <c r="D18" s="4"/>
       <c r="E18" s="2"/>
       <c r="F18" s="3"/>
-      <c r="G18" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H18" s="3"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="6"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
@@ -3299,10 +3454,10 @@
       <c r="Q18" s="2"/>
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
-      <c r="T18" s="2"/>
-      <c r="U18" s="2"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="6"/>
+      <c r="T18" s="3"/>
+      <c r="U18" s="6"/>
+      <c r="V18" s="2"/>
+      <c r="W18" s="2"/>
       <c r="X18" s="2"/>
       <c r="Y18" s="2"/>
       <c r="Z18" s="2"/>
@@ -3311,10 +3466,10 @@
       <c r="AC18" s="2"/>
       <c r="AD18" s="2"/>
       <c r="AE18" s="2"/>
-      <c r="AF18" s="2"/>
-      <c r="AG18" s="2"/>
-      <c r="AH18" s="3"/>
-      <c r="AI18" s="6"/>
+      <c r="AF18" s="3"/>
+      <c r="AG18" s="6"/>
+      <c r="AH18" s="2"/>
+      <c r="AI18" s="2"/>
       <c r="AJ18" s="2"/>
       <c r="AK18" s="2"/>
       <c r="AL18" s="2"/>
@@ -3323,11 +3478,9 @@
       <c r="AO18" s="2"/>
       <c r="AP18" s="2"/>
       <c r="AQ18" s="2"/>
-      <c r="AR18" s="2"/>
-      <c r="AS18" s="2"/>
-      <c r="AT18" s="3"/>
+      <c r="AR18" s="3"/>
     </row>
-    <row r="19" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7">
         <v>46127</v>
       </c>
@@ -3336,14 +3489,11 @@
       <c r="D19" s="4"/>
       <c r="E19" s="2"/>
       <c r="F19" s="3"/>
-      <c r="G19" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H19" s="3"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="6"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
@@ -3352,10 +3502,10 @@
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
       <c r="S19" s="2"/>
-      <c r="T19" s="2"/>
-      <c r="U19" s="2"/>
-      <c r="V19" s="3"/>
-      <c r="W19" s="6"/>
+      <c r="T19" s="3"/>
+      <c r="U19" s="6"/>
+      <c r="V19" s="2"/>
+      <c r="W19" s="2"/>
       <c r="X19" s="2"/>
       <c r="Y19" s="2"/>
       <c r="Z19" s="2"/>
@@ -3364,10 +3514,10 @@
       <c r="AC19" s="2"/>
       <c r="AD19" s="2"/>
       <c r="AE19" s="2"/>
-      <c r="AF19" s="2"/>
-      <c r="AG19" s="2"/>
-      <c r="AH19" s="3"/>
-      <c r="AI19" s="6"/>
+      <c r="AF19" s="3"/>
+      <c r="AG19" s="6"/>
+      <c r="AH19" s="2"/>
+      <c r="AI19" s="2"/>
       <c r="AJ19" s="2"/>
       <c r="AK19" s="2"/>
       <c r="AL19" s="2"/>
@@ -3376,11 +3526,9 @@
       <c r="AO19" s="2"/>
       <c r="AP19" s="2"/>
       <c r="AQ19" s="2"/>
-      <c r="AR19" s="2"/>
-      <c r="AS19" s="2"/>
-      <c r="AT19" s="3"/>
+      <c r="AR19" s="3"/>
     </row>
-    <row r="20" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7">
         <v>46128</v>
       </c>
@@ -3389,14 +3537,11 @@
       <c r="D20" s="4"/>
       <c r="E20" s="2"/>
       <c r="F20" s="3"/>
-      <c r="G20" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H20" s="3"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="6"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
@@ -3405,10 +3550,10 @@
       <c r="Q20" s="2"/>
       <c r="R20" s="2"/>
       <c r="S20" s="2"/>
-      <c r="T20" s="2"/>
-      <c r="U20" s="2"/>
-      <c r="V20" s="3"/>
-      <c r="W20" s="6"/>
+      <c r="T20" s="3"/>
+      <c r="U20" s="6"/>
+      <c r="V20" s="2"/>
+      <c r="W20" s="2"/>
       <c r="X20" s="2"/>
       <c r="Y20" s="2"/>
       <c r="Z20" s="2"/>
@@ -3417,10 +3562,10 @@
       <c r="AC20" s="2"/>
       <c r="AD20" s="2"/>
       <c r="AE20" s="2"/>
-      <c r="AF20" s="2"/>
-      <c r="AG20" s="2"/>
-      <c r="AH20" s="3"/>
-      <c r="AI20" s="6"/>
+      <c r="AF20" s="3"/>
+      <c r="AG20" s="6"/>
+      <c r="AH20" s="2"/>
+      <c r="AI20" s="2"/>
       <c r="AJ20" s="2"/>
       <c r="AK20" s="2"/>
       <c r="AL20" s="2"/>
@@ -3429,11 +3574,9 @@
       <c r="AO20" s="2"/>
       <c r="AP20" s="2"/>
       <c r="AQ20" s="2"/>
-      <c r="AR20" s="2"/>
-      <c r="AS20" s="2"/>
-      <c r="AT20" s="3"/>
+      <c r="AR20" s="3"/>
     </row>
-    <row r="21" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7">
         <v>46129</v>
       </c>
@@ -3442,14 +3585,11 @@
       <c r="D21" s="4"/>
       <c r="E21" s="2"/>
       <c r="F21" s="3"/>
-      <c r="G21" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H21" s="3"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="6"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
@@ -3458,10 +3598,10 @@
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
-      <c r="T21" s="2"/>
-      <c r="U21" s="2"/>
-      <c r="V21" s="3"/>
-      <c r="W21" s="6"/>
+      <c r="T21" s="3"/>
+      <c r="U21" s="6"/>
+      <c r="V21" s="2"/>
+      <c r="W21" s="2"/>
       <c r="X21" s="2"/>
       <c r="Y21" s="2"/>
       <c r="Z21" s="2"/>
@@ -3470,10 +3610,10 @@
       <c r="AC21" s="2"/>
       <c r="AD21" s="2"/>
       <c r="AE21" s="2"/>
-      <c r="AF21" s="2"/>
-      <c r="AG21" s="2"/>
-      <c r="AH21" s="3"/>
-      <c r="AI21" s="6"/>
+      <c r="AF21" s="3"/>
+      <c r="AG21" s="6"/>
+      <c r="AH21" s="2"/>
+      <c r="AI21" s="2"/>
       <c r="AJ21" s="2"/>
       <c r="AK21" s="2"/>
       <c r="AL21" s="2"/>
@@ -3482,11 +3622,9 @@
       <c r="AO21" s="2"/>
       <c r="AP21" s="2"/>
       <c r="AQ21" s="2"/>
-      <c r="AR21" s="2"/>
-      <c r="AS21" s="2"/>
-      <c r="AT21" s="3"/>
+      <c r="AR21" s="3"/>
     </row>
-    <row r="22" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
         <v>46130</v>
       </c>
@@ -3495,14 +3633,11 @@
       <c r="D22" s="4"/>
       <c r="E22" s="2"/>
       <c r="F22" s="3"/>
-      <c r="G22" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H22" s="3"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="6"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
@@ -3511,10 +3646,10 @@
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
       <c r="S22" s="2"/>
-      <c r="T22" s="2"/>
-      <c r="U22" s="2"/>
-      <c r="V22" s="3"/>
-      <c r="W22" s="6"/>
+      <c r="T22" s="3"/>
+      <c r="U22" s="6"/>
+      <c r="V22" s="2"/>
+      <c r="W22" s="2"/>
       <c r="X22" s="2"/>
       <c r="Y22" s="2"/>
       <c r="Z22" s="2"/>
@@ -3523,11 +3658,11 @@
       <c r="AC22" s="2"/>
       <c r="AD22" s="2"/>
       <c r="AE22" s="2"/>
-      <c r="AF22" s="2"/>
-      <c r="AG22" s="2"/>
-      <c r="AH22" s="3"/>
-      <c r="AI22" s="6"/>
-      <c r="AJ22" s="4"/>
+      <c r="AF22" s="3"/>
+      <c r="AG22" s="6"/>
+      <c r="AH22" s="4"/>
+      <c r="AI22" s="2"/>
+      <c r="AJ22" s="2"/>
       <c r="AK22" s="2"/>
       <c r="AL22" s="2"/>
       <c r="AM22" s="2"/>
@@ -3536,10 +3671,8 @@
       <c r="AP22" s="2"/>
       <c r="AQ22" s="2"/>
       <c r="AR22" s="2"/>
-      <c r="AS22" s="2"/>
-      <c r="AT22" s="2"/>
     </row>
-    <row r="23" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7">
         <v>46131</v>
       </c>
@@ -3548,14 +3681,11 @@
       <c r="D23" s="4"/>
       <c r="E23" s="2"/>
       <c r="F23" s="3"/>
-      <c r="G23" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H23" s="3"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="6"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
@@ -3564,10 +3694,10 @@
       <c r="Q23" s="2"/>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
-      <c r="T23" s="2"/>
-      <c r="U23" s="2"/>
-      <c r="V23" s="3"/>
-      <c r="W23" s="6"/>
+      <c r="T23" s="3"/>
+      <c r="U23" s="6"/>
+      <c r="V23" s="2"/>
+      <c r="W23" s="2"/>
       <c r="X23" s="2"/>
       <c r="Y23" s="2"/>
       <c r="Z23" s="2"/>
@@ -3576,11 +3706,11 @@
       <c r="AC23" s="2"/>
       <c r="AD23" s="2"/>
       <c r="AE23" s="2"/>
-      <c r="AF23" s="2"/>
-      <c r="AG23" s="2"/>
-      <c r="AH23" s="3"/>
-      <c r="AI23" s="6"/>
-      <c r="AJ23" s="4"/>
+      <c r="AF23" s="3"/>
+      <c r="AG23" s="6"/>
+      <c r="AH23" s="4"/>
+      <c r="AI23" s="2"/>
+      <c r="AJ23" s="2"/>
       <c r="AK23" s="2"/>
       <c r="AL23" s="2"/>
       <c r="AM23" s="2"/>
@@ -3589,10 +3719,8 @@
       <c r="AP23" s="2"/>
       <c r="AQ23" s="2"/>
       <c r="AR23" s="2"/>
-      <c r="AS23" s="2"/>
-      <c r="AT23" s="2"/>
     </row>
-    <row r="24" spans="1:46" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:44" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
         <v>46132</v>
       </c>
@@ -3601,14 +3729,11 @@
       <c r="D24" s="4"/>
       <c r="E24" s="2"/>
       <c r="F24" s="3"/>
-      <c r="G24" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H24" s="3"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="6"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
@@ -3617,10 +3742,10 @@
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
-      <c r="T24" s="2"/>
-      <c r="U24" s="2"/>
-      <c r="V24" s="3"/>
-      <c r="W24" s="6"/>
+      <c r="T24" s="3"/>
+      <c r="U24" s="6"/>
+      <c r="V24" s="2"/>
+      <c r="W24" s="2"/>
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
       <c r="Z24" s="2"/>
@@ -3629,11 +3754,11 @@
       <c r="AC24" s="2"/>
       <c r="AD24" s="2"/>
       <c r="AE24" s="2"/>
-      <c r="AF24" s="2"/>
-      <c r="AG24" s="2"/>
-      <c r="AH24" s="3"/>
-      <c r="AI24" s="6"/>
-      <c r="AJ24" s="4"/>
+      <c r="AF24" s="3"/>
+      <c r="AG24" s="6"/>
+      <c r="AH24" s="4"/>
+      <c r="AI24" s="2"/>
+      <c r="AJ24" s="2"/>
       <c r="AK24" s="2"/>
       <c r="AL24" s="2"/>
       <c r="AM24" s="2"/>
@@ -3642,10 +3767,8 @@
       <c r="AP24" s="2"/>
       <c r="AQ24" s="2"/>
       <c r="AR24" s="2"/>
-      <c r="AS24" s="2"/>
-      <c r="AT24" s="2"/>
     </row>
-    <row r="25" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7">
         <v>46133</v>
       </c>
@@ -3654,14 +3777,11 @@
       <c r="D25" s="4"/>
       <c r="E25" s="2"/>
       <c r="F25" s="3"/>
-      <c r="G25" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H25" s="3"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="6"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
@@ -3670,10 +3790,10 @@
       <c r="Q25" s="2"/>
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
-      <c r="T25" s="2"/>
-      <c r="U25" s="2"/>
-      <c r="V25" s="3"/>
-      <c r="W25" s="6"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="6"/>
+      <c r="V25" s="2"/>
+      <c r="W25" s="2"/>
       <c r="X25" s="2"/>
       <c r="Y25" s="2"/>
       <c r="Z25" s="2"/>
@@ -3682,11 +3802,11 @@
       <c r="AC25" s="2"/>
       <c r="AD25" s="2"/>
       <c r="AE25" s="2"/>
-      <c r="AF25" s="2"/>
-      <c r="AG25" s="2"/>
-      <c r="AH25" s="3"/>
-      <c r="AI25" s="6"/>
-      <c r="AJ25" s="4"/>
+      <c r="AF25" s="3"/>
+      <c r="AG25" s="6"/>
+      <c r="AH25" s="4"/>
+      <c r="AI25" s="2"/>
+      <c r="AJ25" s="2"/>
       <c r="AK25" s="2"/>
       <c r="AL25" s="2"/>
       <c r="AM25" s="2"/>
@@ -3695,10 +3815,8 @@
       <c r="AP25" s="2"/>
       <c r="AQ25" s="2"/>
       <c r="AR25" s="2"/>
-      <c r="AS25" s="2"/>
-      <c r="AT25" s="2"/>
     </row>
-    <row r="26" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
         <v>46134</v>
       </c>
@@ -3707,14 +3825,11 @@
       <c r="D26" s="4"/>
       <c r="E26" s="2"/>
       <c r="F26" s="3"/>
-      <c r="G26" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H26" s="3"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="6"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
@@ -3723,10 +3838,10 @@
       <c r="Q26" s="2"/>
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
-      <c r="T26" s="2"/>
-      <c r="U26" s="2"/>
-      <c r="V26" s="3"/>
-      <c r="W26" s="6"/>
+      <c r="T26" s="3"/>
+      <c r="U26" s="6"/>
+      <c r="V26" s="2"/>
+      <c r="W26" s="2"/>
       <c r="X26" s="2"/>
       <c r="Y26" s="2"/>
       <c r="Z26" s="2"/>
@@ -3735,11 +3850,11 @@
       <c r="AC26" s="2"/>
       <c r="AD26" s="2"/>
       <c r="AE26" s="2"/>
-      <c r="AF26" s="2"/>
-      <c r="AG26" s="2"/>
-      <c r="AH26" s="3"/>
-      <c r="AI26" s="6"/>
-      <c r="AJ26" s="4"/>
+      <c r="AF26" s="3"/>
+      <c r="AG26" s="6"/>
+      <c r="AH26" s="4"/>
+      <c r="AI26" s="2"/>
+      <c r="AJ26" s="2"/>
       <c r="AK26" s="2"/>
       <c r="AL26" s="2"/>
       <c r="AM26" s="2"/>
@@ -3748,10 +3863,8 @@
       <c r="AP26" s="2"/>
       <c r="AQ26" s="2"/>
       <c r="AR26" s="2"/>
-      <c r="AS26" s="2"/>
-      <c r="AT26" s="2"/>
     </row>
-    <row r="27" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7">
         <v>46135</v>
       </c>
@@ -3760,14 +3873,11 @@
       <c r="D27" s="4"/>
       <c r="E27" s="2"/>
       <c r="F27" s="3"/>
-      <c r="G27" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H27" s="3"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="6"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
@@ -3776,10 +3886,10 @@
       <c r="Q27" s="2"/>
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
-      <c r="T27" s="2"/>
-      <c r="U27" s="2"/>
-      <c r="V27" s="3"/>
-      <c r="W27" s="6"/>
+      <c r="T27" s="3"/>
+      <c r="U27" s="6"/>
+      <c r="V27" s="2"/>
+      <c r="W27" s="2"/>
       <c r="X27" s="2"/>
       <c r="Y27" s="2"/>
       <c r="Z27" s="2"/>
@@ -3788,11 +3898,11 @@
       <c r="AC27" s="2"/>
       <c r="AD27" s="2"/>
       <c r="AE27" s="2"/>
-      <c r="AF27" s="2"/>
-      <c r="AG27" s="2"/>
-      <c r="AH27" s="3"/>
-      <c r="AI27" s="6"/>
-      <c r="AJ27" s="4"/>
+      <c r="AF27" s="3"/>
+      <c r="AG27" s="6"/>
+      <c r="AH27" s="4"/>
+      <c r="AI27" s="2"/>
+      <c r="AJ27" s="2"/>
       <c r="AK27" s="2"/>
       <c r="AL27" s="2"/>
       <c r="AM27" s="2"/>
@@ -3801,10 +3911,8 @@
       <c r="AP27" s="2"/>
       <c r="AQ27" s="2"/>
       <c r="AR27" s="2"/>
-      <c r="AS27" s="2"/>
-      <c r="AT27" s="2"/>
     </row>
-    <row r="28" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
         <v>46136</v>
       </c>
@@ -3813,14 +3921,11 @@
       <c r="D28" s="4"/>
       <c r="E28" s="2"/>
       <c r="F28" s="3"/>
-      <c r="G28" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H28" s="3"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="6"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
@@ -3829,10 +3934,10 @@
       <c r="Q28" s="2"/>
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
-      <c r="T28" s="2"/>
-      <c r="U28" s="2"/>
-      <c r="V28" s="3"/>
-      <c r="W28" s="6"/>
+      <c r="T28" s="3"/>
+      <c r="U28" s="6"/>
+      <c r="V28" s="2"/>
+      <c r="W28" s="2"/>
       <c r="X28" s="2"/>
       <c r="Y28" s="2"/>
       <c r="Z28" s="2"/>
@@ -3841,11 +3946,11 @@
       <c r="AC28" s="2"/>
       <c r="AD28" s="2"/>
       <c r="AE28" s="2"/>
-      <c r="AF28" s="2"/>
-      <c r="AG28" s="2"/>
-      <c r="AH28" s="3"/>
-      <c r="AI28" s="6"/>
-      <c r="AJ28" s="4"/>
+      <c r="AF28" s="3"/>
+      <c r="AG28" s="6"/>
+      <c r="AH28" s="4"/>
+      <c r="AI28" s="2"/>
+      <c r="AJ28" s="2"/>
       <c r="AK28" s="2"/>
       <c r="AL28" s="2"/>
       <c r="AM28" s="2"/>
@@ -3854,10 +3959,8 @@
       <c r="AP28" s="2"/>
       <c r="AQ28" s="2"/>
       <c r="AR28" s="2"/>
-      <c r="AS28" s="2"/>
-      <c r="AT28" s="2"/>
     </row>
-    <row r="29" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7">
         <v>46137</v>
       </c>
@@ -3866,14 +3969,11 @@
       <c r="D29" s="4"/>
       <c r="E29" s="2"/>
       <c r="F29" s="3"/>
-      <c r="G29" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H29" s="3"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="5"/>
-      <c r="K29" s="6"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
@@ -3882,10 +3982,10 @@
       <c r="Q29" s="2"/>
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
-      <c r="T29" s="2"/>
-      <c r="U29" s="2"/>
-      <c r="V29" s="3"/>
-      <c r="W29" s="6"/>
+      <c r="T29" s="3"/>
+      <c r="U29" s="6"/>
+      <c r="V29" s="2"/>
+      <c r="W29" s="2"/>
       <c r="X29" s="2"/>
       <c r="Y29" s="2"/>
       <c r="Z29" s="2"/>
@@ -3894,11 +3994,11 @@
       <c r="AC29" s="2"/>
       <c r="AD29" s="2"/>
       <c r="AE29" s="2"/>
-      <c r="AF29" s="2"/>
-      <c r="AG29" s="2"/>
-      <c r="AH29" s="3"/>
-      <c r="AI29" s="6"/>
-      <c r="AJ29" s="4"/>
+      <c r="AF29" s="3"/>
+      <c r="AG29" s="6"/>
+      <c r="AH29" s="4"/>
+      <c r="AI29" s="2"/>
+      <c r="AJ29" s="2"/>
       <c r="AK29" s="2"/>
       <c r="AL29" s="2"/>
       <c r="AM29" s="2"/>
@@ -3907,10 +4007,8 @@
       <c r="AP29" s="2"/>
       <c r="AQ29" s="2"/>
       <c r="AR29" s="2"/>
-      <c r="AS29" s="2"/>
-      <c r="AT29" s="2"/>
     </row>
-    <row r="30" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
         <v>46138</v>
       </c>
@@ -3929,169 +4027,164 @@
       <c r="E30" s="2">
         <v>77.91</v>
       </c>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>91.807485900009425</v>
-      </c>
-      <c r="H30" s="3">
+      <c r="F30" s="3">
         <f>[1]PR_Calc!$AA$111</f>
         <v>2585.0777272727278</v>
       </c>
-      <c r="I30" s="2">
+      <c r="G30" s="2">
         <f>[1]PR_Calc!AN$111</f>
         <v>2575.6800000000003</v>
       </c>
-      <c r="J30" s="5">
+      <c r="H30" s="5">
         <f>[1]PR_Calc!BA$111</f>
         <v>2630.3231818181821</v>
       </c>
-      <c r="K30" s="6">
+      <c r="I30" s="6">
         <f>[1]PR_Calc!O$111</f>
         <v>0.85822998958753727</v>
       </c>
-      <c r="L30" s="2">
+      <c r="J30" s="2">
         <f>[1]PR_Calc!P$111</f>
         <v>0.8569062313765915</v>
       </c>
-      <c r="M30" s="2">
+      <c r="K30" s="2">
         <f>[1]PR_Calc!Q$111</f>
         <v>0.85982296382707624</v>
       </c>
-      <c r="N30" s="2">
+      <c r="L30" s="2">
         <f>[1]PR_Calc!R$111</f>
         <v>0.85966671030294295</v>
       </c>
-      <c r="O30" s="2">
+      <c r="M30" s="2">
         <f>[1]PR_Calc!S$111</f>
         <v>0.85880359559820818</v>
       </c>
-      <c r="P30" s="2">
+      <c r="N30" s="2">
         <f>[1]PR_Calc!T$111</f>
         <v>0.85674997785245799</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="O30" s="2">
         <f>[1]PR_Calc!U$111</f>
         <v>0.85532881484724654</v>
       </c>
-      <c r="R30" s="2">
+      <c r="P30" s="2">
         <f>[1]PR_Calc!V$111</f>
         <v>0.83395488557588593</v>
       </c>
-      <c r="S30" s="2">
+      <c r="Q30" s="2">
         <f>[1]PR_Calc!W$111</f>
         <v>0.83188379849203453</v>
       </c>
-      <c r="T30" s="2">
+      <c r="R30" s="2">
         <f>[1]PR_Calc!X$111</f>
         <v>0.82917928614886016</v>
       </c>
-      <c r="U30" s="2">
+      <c r="S30" s="2">
         <f>[1]PR_Calc!Y$111</f>
         <v>0.83039631670328851</v>
       </c>
-      <c r="V30" s="2">
+      <c r="T30" s="2">
         <f>[1]PR_Calc!Z$111</f>
         <v>0.85632586114409648</v>
       </c>
-      <c r="W30" s="6">
+      <c r="U30" s="6">
         <f>[1]PR_Calc!AB$111</f>
         <v>0.88474827088900154</v>
       </c>
-      <c r="X30" s="2">
+      <c r="V30" s="2">
         <f>[1]PR_Calc!AC$111</f>
         <v>0.85369931380985831</v>
       </c>
-      <c r="Y30" s="2">
+      <c r="W30" s="2">
         <f>[1]PR_Calc!AD$111</f>
         <v>0.8526501830049642</v>
       </c>
-      <c r="Z30" s="2">
+      <c r="X30" s="2">
         <f>[1]PR_Calc!AE$111</f>
         <v>0.88508345418566814</v>
       </c>
-      <c r="AA30" s="2">
+      <c r="Y30" s="2">
         <f>[1]PR_Calc!AF$111</f>
         <v>0.88811569377644273</v>
       </c>
-      <c r="AB30" s="2">
+      <c r="Z30" s="2">
         <f>[1]PR_Calc!AG$111</f>
         <v>0.82170629151640495</v>
       </c>
-      <c r="AC30" s="2">
+      <c r="AA30" s="2">
         <f>[1]PR_Calc!AH$111</f>
         <v>0.85136295159186715</v>
       </c>
-      <c r="AD30" s="2">
+      <c r="AB30" s="2">
         <f>[1]PR_Calc!AI$111</f>
         <v>0.82036115248256303</v>
       </c>
-      <c r="AE30" s="2">
+      <c r="AC30" s="2">
         <f>[1]PR_Calc!AJ$111</f>
         <v>0.81996970990657769</v>
       </c>
-      <c r="AF30" s="2">
+      <c r="AD30" s="2">
         <f>[1]PR_Calc!AK$111</f>
         <v>0.84956231574233276</v>
       </c>
-      <c r="AG30" s="2">
+      <c r="AE30" s="2">
         <f>[1]PR_Calc!AL$111</f>
         <v>0.81830429967420215</v>
       </c>
-      <c r="AH30" s="2">
+      <c r="AF30" s="2">
         <f>[1]PR_Calc!AM$111</f>
         <v>0.81933628464725528</v>
       </c>
-      <c r="AI30" s="6">
+      <c r="AG30" s="6">
         <f>[1]PR_Calc!AO$111</f>
         <v>0.83918598181860449</v>
       </c>
-      <c r="AJ30" s="4">
+      <c r="AH30" s="4">
         <f>[1]PR_Calc!AP$111</f>
         <v>0.83783372564701741</v>
       </c>
-      <c r="AK30" s="2">
+      <c r="AI30" s="2">
         <f>[1]PR_Calc!AQ$111</f>
         <v>0.83652417230190146</v>
       </c>
-      <c r="AL30" s="2">
+      <c r="AJ30" s="2">
         <f>[1]PR_Calc!AR$111</f>
         <v>0.83746363448426697</v>
       </c>
-      <c r="AM30" s="2">
+      <c r="AK30" s="2">
         <f>[1]PR_Calc!AS$111</f>
         <v>0.83758462582593529</v>
       </c>
-      <c r="AN30" s="2">
+      <c r="AL30" s="2">
         <f>[1]PR_Calc!AT$111</f>
         <v>0.84009697544998896</v>
       </c>
-      <c r="AO30" s="2">
+      <c r="AM30" s="2">
         <f>[1]PR_Calc!AU$111</f>
         <v>0.84015908865212896</v>
       </c>
-      <c r="AP30" s="2">
+      <c r="AN30" s="2">
         <f>[1]PR_Calc!AV$111</f>
         <v>0.83466659935040544</v>
       </c>
-      <c r="AQ30" s="2">
+      <c r="AO30" s="2">
         <f>[1]PR_Calc!AW$111</f>
         <v>0.83826787104947442</v>
       </c>
-      <c r="AR30" s="2">
+      <c r="AP30" s="2">
         <f>[1]PR_Calc!AX$111</f>
         <v>0.83846003376859424</v>
       </c>
-      <c r="AS30" s="2">
+      <c r="AQ30" s="2">
         <f>[1]PR_Calc!AY$111</f>
         <v>0.83796895126417592</v>
       </c>
-      <c r="AT30" s="2">
+      <c r="AR30" s="2">
         <f>[1]PR_Calc!AZ$111</f>
         <v>0.90562317480697996</v>
       </c>
     </row>
-    <row r="31" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7">
         <v>46139</v>
       </c>
@@ -4100,14 +4193,11 @@
       <c r="D31" s="4"/>
       <c r="E31" s="2"/>
       <c r="F31" s="3"/>
-      <c r="G31" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H31" s="3"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="5"/>
-      <c r="K31" s="6"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
@@ -4116,10 +4206,10 @@
       <c r="Q31" s="2"/>
       <c r="R31" s="2"/>
       <c r="S31" s="2"/>
-      <c r="T31" s="2"/>
-      <c r="U31" s="2"/>
-      <c r="V31" s="3"/>
-      <c r="W31" s="6"/>
+      <c r="T31" s="3"/>
+      <c r="U31" s="6"/>
+      <c r="V31" s="2"/>
+      <c r="W31" s="2"/>
       <c r="X31" s="2"/>
       <c r="Y31" s="2"/>
       <c r="Z31" s="2"/>
@@ -4128,11 +4218,11 @@
       <c r="AC31" s="2"/>
       <c r="AD31" s="2"/>
       <c r="AE31" s="2"/>
-      <c r="AF31" s="2"/>
-      <c r="AG31" s="2"/>
-      <c r="AH31" s="3"/>
-      <c r="AI31" s="6"/>
-      <c r="AJ31" s="4"/>
+      <c r="AF31" s="3"/>
+      <c r="AG31" s="6"/>
+      <c r="AH31" s="4"/>
+      <c r="AI31" s="2"/>
+      <c r="AJ31" s="2"/>
       <c r="AK31" s="2"/>
       <c r="AL31" s="2"/>
       <c r="AM31" s="2"/>
@@ -4141,10 +4231,8 @@
       <c r="AP31" s="2"/>
       <c r="AQ31" s="2"/>
       <c r="AR31" s="2"/>
-      <c r="AS31" s="2"/>
-      <c r="AT31" s="2"/>
     </row>
-    <row r="32" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7">
         <v>46140</v>
       </c>
@@ -4153,14 +4241,11 @@
       <c r="D32" s="4"/>
       <c r="E32" s="2"/>
       <c r="F32" s="3"/>
-      <c r="G32" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H32" s="3"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="5"/>
-      <c r="K32" s="6"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
@@ -4169,10 +4254,10 @@
       <c r="Q32" s="2"/>
       <c r="R32" s="2"/>
       <c r="S32" s="2"/>
-      <c r="T32" s="2"/>
-      <c r="U32" s="2"/>
-      <c r="V32" s="3"/>
-      <c r="W32" s="6"/>
+      <c r="T32" s="3"/>
+      <c r="U32" s="6"/>
+      <c r="V32" s="2"/>
+      <c r="W32" s="2"/>
       <c r="X32" s="2"/>
       <c r="Y32" s="2"/>
       <c r="Z32" s="2"/>
@@ -4181,11 +4266,11 @@
       <c r="AC32" s="2"/>
       <c r="AD32" s="2"/>
       <c r="AE32" s="2"/>
-      <c r="AF32" s="2"/>
-      <c r="AG32" s="2"/>
-      <c r="AH32" s="3"/>
-      <c r="AI32" s="6"/>
-      <c r="AJ32" s="4"/>
+      <c r="AF32" s="3"/>
+      <c r="AG32" s="6"/>
+      <c r="AH32" s="4"/>
+      <c r="AI32" s="2"/>
+      <c r="AJ32" s="2"/>
       <c r="AK32" s="2"/>
       <c r="AL32" s="2"/>
       <c r="AM32" s="2"/>
@@ -4194,10 +4279,8 @@
       <c r="AP32" s="2"/>
       <c r="AQ32" s="2"/>
       <c r="AR32" s="2"/>
-      <c r="AS32" s="2"/>
-      <c r="AT32" s="2"/>
     </row>
-    <row r="33" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7">
         <v>46141</v>
       </c>
@@ -4206,14 +4289,11 @@
       <c r="D33" s="4"/>
       <c r="E33" s="2"/>
       <c r="F33" s="3"/>
-      <c r="G33" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H33" s="3"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="6"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
@@ -4222,10 +4302,10 @@
       <c r="Q33" s="2"/>
       <c r="R33" s="2"/>
       <c r="S33" s="2"/>
-      <c r="T33" s="2"/>
-      <c r="U33" s="2"/>
-      <c r="V33" s="3"/>
-      <c r="W33" s="6"/>
+      <c r="T33" s="3"/>
+      <c r="U33" s="6"/>
+      <c r="V33" s="2"/>
+      <c r="W33" s="2"/>
       <c r="X33" s="2"/>
       <c r="Y33" s="2"/>
       <c r="Z33" s="2"/>
@@ -4234,10 +4314,10 @@
       <c r="AC33" s="2"/>
       <c r="AD33" s="2"/>
       <c r="AE33" s="2"/>
-      <c r="AF33" s="2"/>
-      <c r="AG33" s="2"/>
-      <c r="AH33" s="3"/>
-      <c r="AI33" s="6"/>
+      <c r="AF33" s="3"/>
+      <c r="AG33" s="6"/>
+      <c r="AH33" s="2"/>
+      <c r="AI33" s="2"/>
       <c r="AJ33" s="2"/>
       <c r="AK33" s="2"/>
       <c r="AL33" s="2"/>
@@ -4246,11 +4326,9 @@
       <c r="AO33" s="2"/>
       <c r="AP33" s="2"/>
       <c r="AQ33" s="2"/>
-      <c r="AR33" s="2"/>
-      <c r="AS33" s="2"/>
-      <c r="AT33" s="3"/>
+      <c r="AR33" s="3"/>
     </row>
-    <row r="34" spans="1:46" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7">
         <v>46142</v>
       </c>
@@ -4259,14 +4337,11 @@
       <c r="D34" s="4"/>
       <c r="E34" s="2"/>
       <c r="F34" s="3"/>
-      <c r="G34" s="3" t="e">
-        <f>(TabellaAPRL2026[[#This Row],[Colonna11]]-SUM(TabellaAPRL2026[[#This Row],[Colonna13]:[Colonna15]]))/TabellaAPRL2026[[#This Row],[Colonna11]]*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H34" s="3"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="5"/>
-      <c r="K34" s="6"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
       <c r="L34" s="2"/>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
@@ -4275,10 +4350,10 @@
       <c r="Q34" s="2"/>
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
-      <c r="T34" s="2"/>
-      <c r="U34" s="2"/>
-      <c r="V34" s="3"/>
-      <c r="W34" s="6"/>
+      <c r="T34" s="3"/>
+      <c r="U34" s="6"/>
+      <c r="V34" s="2"/>
+      <c r="W34" s="2"/>
       <c r="X34" s="2"/>
       <c r="Y34" s="2"/>
       <c r="Z34" s="2"/>
@@ -4287,10 +4362,10 @@
       <c r="AC34" s="2"/>
       <c r="AD34" s="2"/>
       <c r="AE34" s="2"/>
-      <c r="AF34" s="2"/>
-      <c r="AG34" s="2"/>
-      <c r="AH34" s="3"/>
-      <c r="AI34" s="6"/>
+      <c r="AF34" s="3"/>
+      <c r="AG34" s="6"/>
+      <c r="AH34" s="2"/>
+      <c r="AI34" s="2"/>
       <c r="AJ34" s="2"/>
       <c r="AK34" s="2"/>
       <c r="AL34" s="2"/>
@@ -4299,11 +4374,9 @@
       <c r="AO34" s="2"/>
       <c r="AP34" s="2"/>
       <c r="AQ34" s="2"/>
-      <c r="AR34" s="2"/>
-      <c r="AS34" s="2"/>
-      <c r="AT34" s="3"/>
+      <c r="AR34" s="3"/>
     </row>
-    <row r="35" spans="1:46" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:44" x14ac:dyDescent="0.25">
       <c r="B35" s="11"/>
       <c r="C35" s="11"/>
       <c r="D35" s="19">
@@ -4314,18 +4387,12 @@
         <f>AVERAGE(E5:E34)</f>
         <v>77.91</v>
       </c>
-      <c r="F35" s="30" t="e">
-        <f>AVERAGE(F5:F34)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G35" s="30" t="e">
-        <f>SUMIF(G5:G34,"&lt;&gt;100")/COUNTIF(G5:G34,"&lt;&gt;100")</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H35" s="12"/>
-      <c r="I35" s="11"/>
-      <c r="J35" s="13"/>
-      <c r="K35" s="14"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="13"/>
+      <c r="I35" s="14"/>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15"/>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
       <c r="N35" s="15"/>
@@ -4334,10 +4401,10 @@
       <c r="Q35" s="15"/>
       <c r="R35" s="15"/>
       <c r="S35" s="15"/>
-      <c r="T35" s="15"/>
-      <c r="U35" s="15"/>
-      <c r="V35" s="16"/>
-      <c r="W35" s="17"/>
+      <c r="T35" s="16"/>
+      <c r="U35" s="17"/>
+      <c r="V35" s="18"/>
+      <c r="W35" s="18"/>
       <c r="X35" s="18"/>
       <c r="Y35" s="18"/>
       <c r="Z35" s="18"/>
@@ -4347,9 +4414,9 @@
       <c r="AD35" s="18"/>
       <c r="AE35" s="18"/>
       <c r="AF35" s="18"/>
-      <c r="AG35" s="18"/>
+      <c r="AG35" s="17"/>
       <c r="AH35" s="18"/>
-      <c r="AI35" s="17"/>
+      <c r="AI35" s="18"/>
       <c r="AJ35" s="18"/>
       <c r="AK35" s="18"/>
       <c r="AL35" s="18"/>
@@ -4359,15 +4426,13 @@
       <c r="AP35" s="18"/>
       <c r="AQ35" s="18"/>
       <c r="AR35" s="18"/>
-      <c r="AS35" s="18"/>
-      <c r="AT35" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:AT1"/>
+    <mergeCell ref="A1:AR1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D5:G34">
-    <cfRule type="cellIs" dxfId="46" priority="1" operator="greaterThan">
+  <conditionalFormatting sqref="D5:E34">
+    <cfRule type="cellIs" dxfId="54" priority="1" operator="greaterThan">
       <formula>100</formula>
     </cfRule>
     <cfRule type="colorScale" priority="13">
@@ -4379,7 +4444,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:AT34">
+  <conditionalFormatting sqref="I5:AR34">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="num" val="0"/>

</xml_diff>